<commit_message>
İK/kariyer e-posta sütunu ve kullanıcının 24 firması eklendi
- Toplayıcı artık genel kurumsal adres ile İK adresini (ik@, kariyer@,
  career@, cv@, insankaynaklari@, hr@, jobs@) ayrı sütunlarda topluyor;
  /kariyer, /careers, /insan-kaynaklari gibi İK sayfaları da taranıyor.
- --varyant-uret bayrağı, siteden doğrulanamayan firmalar için istenen
  dört varyantı üretiyor. Üretilen adresler 'Doğrulama' sütununda
  'üretildi – doğrulanmadı' olarak işaretlenip kırmızı gösteriliyor.
- Tohum listesine 24 firma eklendi; obss.tech, iyzico.com ve marti.tech
  listede zaten olduğu için alan adına göre tekilleştirildi.
- E-postalar hâlâ doğrulanmadı: egress politikası bu firmaların
  sitelerini de reddediyor.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016m9M3fsJ1qn42BpGV3myHC
</commit_message>
<xml_diff>
--- a/istanbul_yazilim_sirketleri.xlsx
+++ b/istanbul_yazilim_sirketleri.xlsx
@@ -11,7 +11,7 @@
     <sheet name="OKUBENI" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Şirketler'!$A$1:$E$70</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Şirketler'!$A$1:$G$94</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -36,6 +36,11 @@
     </font>
     <font>
       <name val="Arial"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00C00000"/>
       <sz val="10"/>
     </font>
     <font>
@@ -69,7 +74,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -78,6 +83,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -448,14 +456,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E70"/>
+  <dimension ref="A1:G94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="46" customWidth="1" min="5" max="5"/>
+    <col width="46" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -476,12 +486,22 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>İK / Kariyer E-postası</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>Sektör / Faaliyet Alanı</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Kaynak</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Doğrulama</t>
         </is>
       </c>
     </row>
@@ -497,14 +517,24 @@
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr"/>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>ik@akinon.com, kariyer@akinon.com, career@akinon.com, cv@akinon.com</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>E-ticaret yazılım platformu</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Ön liste (doğrulanmadı)</t>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
     </row>
@@ -520,14 +550,24 @@
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr"/>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>ik@appcent.mobi, kariyer@appcent.mobi, career@appcent.mobi, cv@appcent.mobi</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>Mobil uygulama geliştirme</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>Ön liste (doğrulanmadı)</t>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
     </row>
@@ -543,1537 +583,2971 @@
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr"/>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>ik@armut.com, kariyer@armut.com, career@armut.com, cv@armut.com</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>Hizmet pazaryeri</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>Ön liste (doğrulanmadı)</t>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Berqnet</t>
+          <t>ATP Teknoloji</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>https://www.berqnet.com</t>
+          <t>https://www.atptech.com</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr"/>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>Siber güvenlik / güvenlik duvarı</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>Ön liste (doğrulanmadı)</t>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>ik@atptech.com, kariyer@atptech.com, career@atptech.com, cv@atptech.com</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr"/>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Kullanıcı listesi (05.08.2026)</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>BiTaksi</t>
+          <t>AVDCG</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>https://bitaksi.com</t>
+          <t>https://avdcg.com</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr"/>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>Mobilite / mobil uygulama</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>Ön liste (doğrulanmadı)</t>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>ik@avdcg.com, kariyer@avdcg.com, career@avdcg.com, cv@avdcg.com</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr"/>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Kullanıcı listesi (05.08.2026)</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Bitexen</t>
+          <t>Berqnet</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>https://www.bitexen.com</t>
+          <t>https://www.berqnet.com</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr"/>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>Kripto varlık platformu</t>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>ik@berqnet.com, kariyer@berqnet.com, career@berqnet.com, cv@berqnet.com</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Siber güvenlik / güvenlik duvarı</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>BtcTurk</t>
+          <t>Bimser Çözüm</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>https://www.btcturk.com</t>
+          <t>https://bimser.com</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr"/>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>Kripto varlık platformu</t>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>ik@bimser.com, kariyer@bimser.com, career@bimser.com, cv@bimser.com</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Kurumsal yazılım (QDMS / eBA)</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Kullanıcı listesi (05.08.2026)</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Codeway</t>
+          <t>BiTaksi</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>https://codeway.co</t>
+          <t>https://bitaksi.com</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr"/>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>Mobil uygulama geliştirme</t>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>ik@bitaksi.com, kariyer@bitaksi.com, career@bitaksi.com, cv@bitaksi.com</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Mobilite / mobil uygulama</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Colendi</t>
+          <t>Bitexen</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>https://www.colendi.com</t>
+          <t>https://www.bitexen.com</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr"/>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>Fintech / dijital bankacılık</t>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>ik@bitexen.com, kariyer@bitexen.com, career@bitexen.com, cv@bitexen.com</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Kripto varlık platformu</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Commencis</t>
+          <t>Blue Arf</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>https://www.commencis.com</t>
+          <t>https://www.bluearf.com</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr"/>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>Dijital ürün / yazılım geliştirme</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>Ön liste (doğrulanmadı)</t>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>ik@bluearf.com, kariyer@bluearf.com, career@bluearf.com, cv@bluearf.com</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Kullanıcı listesi (05.08.2026)</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>CPM Yazılım</t>
+          <t>BtcTurk</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>https://www.cpm.com.tr</t>
+          <t>https://www.btcturk.com</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr"/>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>Sigortacılık yazılımı</t>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>ik@btcturk.com, kariyer@btcturk.com, career@btcturk.com, cv@btcturk.com</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Kripto varlık platformu</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Craftgate</t>
+          <t>Chippin</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>https://craftgate.io</t>
+          <t>https://chippin.com</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr"/>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>Fintech / ödeme altyapısı</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>Ön liste (doğrulanmadı)</t>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>ik@chippin.com, kariyer@chippin.com, career@chippin.com, cv@chippin.com</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr"/>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Kullanıcı listesi (05.08.2026)</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Detaysoft</t>
+          <t>Codevo</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>https://www.detaysoft.com</t>
+          <t>https://codevo.com.tr</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr"/>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>SAP danışmanlık / kurumsal yazılım</t>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>ik@codevo.com.tr, kariyer@codevo.com.tr, career@codevo.com.tr, cv@codevo.com.tr</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Yazılım geliştirme</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Kullanıcı listesi (05.08.2026)</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Digital Planet</t>
+          <t>Codeway</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>https://www.digitalplanet.com.tr</t>
+          <t>https://codeway.co</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr"/>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>e-Dönüşüm çözümleri</t>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>ik@codeway.co, kariyer@codeway.co, career@codeway.co, cv@codeway.co</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Mobil uygulama geliştirme</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Doğuş Teknoloji</t>
+          <t>Colendi</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>https://www.d-teknoloji.com.tr</t>
+          <t>https://www.colendi.com</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr"/>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>BT hizmetleri</t>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>ik@colendi.com, kariyer@colendi.com, career@colendi.com, cv@colendi.com</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Fintech / dijital bankacılık</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Dream Games</t>
+          <t>Commencis</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>https://www.dreamgames.com</t>
+          <t>https://www.commencis.com</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr"/>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>Mobil oyun</t>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>ik@commencis.com, kariyer@commencis.com, career@commencis.com, cv@commencis.com</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Dijital ürün / yazılım geliştirme</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Etiya</t>
+          <t>CPM Yazılım</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>https://www.etiya.com</t>
+          <t>https://www.cpm.com.tr</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr"/>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>Telekom yazılımı / BSS</t>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>ik@cpm.com.tr, kariyer@cpm.com.tr, career@cpm.com.tr, cv@cpm.com.tr</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Sigortacılık yazılımı</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Experteam</t>
+          <t>Craftgate</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>https://www.experteam.com.tr</t>
+          <t>https://craftgate.io</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr"/>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>SAP danışmanlık</t>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>ik@craftgate.io, kariyer@craftgate.io, career@craftgate.io, cv@craftgate.io</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Fintech / ödeme altyapısı</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Figopara</t>
+          <t>CRS Soft</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>https://www.figopara.com</t>
+          <t>https://www.crssoft.com</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr"/>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>Fintech / tedarik zinciri finansmanı</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
-          <t>Ön liste (doğrulanmadı)</t>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>ik@crssoft.com, kariyer@crssoft.com, career@crssoft.com, cv@crssoft.com</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr"/>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Kullanıcı listesi (05.08.2026)</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Getir</t>
+          <t>Detaysoft</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>https://getir.com</t>
+          <t>https://www.detaysoft.com</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr"/>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t>Hızlı ticaret / mobil uygulama</t>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>ik@detaysoft.com, kariyer@detaysoft.com, career@detaysoft.com, cv@detaysoft.com</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>SAP danışmanlık / kurumsal yazılım</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Gram Games</t>
+          <t>Digital Planet</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>https://www.gramgames.com</t>
+          <t>https://www.digitalplanet.com.tr</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr"/>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>Mobil oyun</t>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>ik@digitalplanet.com.tr, kariyer@digitalplanet.com.tr, career@digitalplanet.com.tr, cv@digitalplanet.com.tr</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>e-Dönüşüm çözümleri</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Hepsiburada</t>
+          <t>Dijital Kurye</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>https://www.hepsiburada.com</t>
+          <t>https://dijitalkurye.com.tr</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr"/>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t>E-ticaret platformu</t>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>ik@dijitalkurye.com.tr, kariyer@dijitalkurye.com.tr, career@dijitalkurye.com.tr, cv@dijitalkurye.com.tr</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Dijital ajans</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>Kullanıcı listesi (05.08.2026)</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>IAS - Canias ERP</t>
+          <t>Doğuş Teknoloji</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>https://www.caniaserp.com</t>
+          <t>https://www.d-teknoloji.com.tr</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr"/>
-      <c r="D24" s="2" t="inlineStr">
-        <is>
-          <t>ERP yazılımı</t>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>ik@d-teknoloji.com.tr, kariyer@d-teknoloji.com.tr, career@d-teknoloji.com.tr, cv@d-teknoloji.com.tr</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>BT hizmetleri</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>IdeaSoft</t>
+          <t>Dream Games</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>https://www.ideasoft.com.tr</t>
+          <t>https://www.dreamgames.com</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr"/>
-      <c r="D25" s="2" t="inlineStr">
-        <is>
-          <t>E-ticaret altyapı yazılımı</t>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>ik@dreamgames.com, kariyer@dreamgames.com, career@dreamgames.com, cv@dreamgames.com</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Mobil oyun</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>ininal</t>
+          <t>Etiya</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>https://www.ininal.com</t>
+          <t>https://www.etiya.com</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr"/>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>Fintech / ön ödemeli kart</t>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>ik@etiya.com, kariyer@etiya.com, career@etiya.com, cv@etiya.com</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Telekom yazılımı / BSS</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Innova Bilişim</t>
+          <t>Experteam</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>https://www.innova.com.tr</t>
+          <t>https://www.experteam.com.tr</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr"/>
-      <c r="D27" s="2" t="inlineStr">
-        <is>
-          <t>BT çözümleri / sistem entegrasyonu</t>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>ik@experteam.com.tr, kariyer@experteam.com.tr, career@experteam.com.tr, cv@experteam.com.tr</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>SAP danışmanlık</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Insider</t>
+          <t>Figopara</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>https://useinsider.com</t>
+          <t>https://www.figopara.com</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr"/>
-      <c r="D28" s="2" t="inlineStr">
-        <is>
-          <t>Pazarlama teknolojileri / SaaS</t>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>ik@figopara.com, kariyer@figopara.com, career@figopara.com, cv@figopara.com</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Fintech / tedarik zinciri finansmanı</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Intertech</t>
+          <t>Getir</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>https://www.intertech.com.tr</t>
+          <t>https://getir.com</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr"/>
-      <c r="D29" s="2" t="inlineStr">
-        <is>
-          <t>Bankacılık teknolojileri</t>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>ik@getir.com, kariyer@getir.com, career@getir.com, cv@getir.com</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Hızlı ticaret / mobil uygulama</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>iyzico</t>
+          <t>Gram Games</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>https://www.iyzico.com</t>
+          <t>https://www.gramgames.com</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr"/>
-      <c r="D30" s="2" t="inlineStr">
-        <is>
-          <t>Fintech / ödeme sistemleri</t>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>ik@gramgames.com, kariyer@gramgames.com, career@gramgames.com, cv@gramgames.com</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Mobil oyun</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>İzibiz</t>
+          <t>Grid Studio</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>https://www.izibiz.com.tr</t>
+          <t>https://gridstudio.ai</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr"/>
-      <c r="D31" s="2" t="inlineStr">
-        <is>
-          <t>e-Fatura / e-dönüşüm</t>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>ik@gridstudio.ai, kariyer@gridstudio.ai, career@gridstudio.ai, cv@gridstudio.ai</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Yapay zeka</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>Kullanıcı listesi (05.08.2026)</t>
+        </is>
+      </c>
+      <c r="G31" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Kariyer.net</t>
+          <t>Hepsiburada</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>https://www.kariyer.net</t>
+          <t>https://www.hepsiburada.com</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr"/>
-      <c r="D32" s="2" t="inlineStr">
-        <is>
-          <t>İK teknolojileri</t>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>ik@hepsiburada.com, kariyer@hepsiburada.com, career@hepsiburada.com, cv@hepsiburada.com</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>E-ticaret platformu</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G32" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>KoçSistem</t>
+          <t>HireFeed</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>https://www.kocsistem.com.tr</t>
+          <t>https://www.hirefeed.co.in</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr"/>
-      <c r="D33" s="2" t="inlineStr">
-        <is>
-          <t>BT hizmetleri / sistem entegrasyonu</t>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>ik@co.in, kariyer@co.in, career@co.in, cv@co.in</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>İK teknolojileri</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>Kullanıcı listesi (05.08.2026)</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Kron Technologies</t>
+          <t>IAS - Canias ERP</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>https://krontech.com</t>
+          <t>https://www.caniaserp.com</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr"/>
-      <c r="D34" s="2" t="inlineStr">
-        <is>
-          <t>Siber güvenlik / erişim yönetimi</t>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>ik@caniaserp.com, kariyer@caniaserp.com, career@caniaserp.com, cv@caniaserp.com</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>ERP yazılımı</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G34" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Link Bilgisayar</t>
+          <t>IdeaSoft</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkbilgisayar.com.tr</t>
+          <t>https://www.ideasoft.com.tr</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr"/>
-      <c r="D35" s="2" t="inlineStr">
-        <is>
-          <t>Ticari yazılım</t>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>ik@ideasoft.com.tr, kariyer@ideasoft.com.tr, career@ideasoft.com.tr, cv@ideasoft.com.tr</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>E-ticaret altyapı yazılımı</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G35" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Martı</t>
+          <t>ininal</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>https://www.marti.tech</t>
+          <t>https://www.ininal.com</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr"/>
-      <c r="D36" s="2" t="inlineStr">
-        <is>
-          <t>Mobilite teknolojileri</t>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>ik@ininal.com, kariyer@ininal.com, career@ininal.com, cv@ininal.com</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Fintech / ön ödemeli kart</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G36" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Midas</t>
+          <t>Innova Bilişim</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>https://www.getmidas.com</t>
+          <t>https://www.innova.com.tr</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr"/>
-      <c r="D37" s="2" t="inlineStr">
-        <is>
-          <t>Fintech / yatırım platformu</t>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>ik@innova.com.tr, kariyer@innova.com.tr, career@innova.com.tr, cv@innova.com.tr</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>BT çözümleri / sistem entegrasyonu</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G37" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Mikro Yazılım</t>
+          <t>Insider</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>https://www.mikro.com.tr</t>
+          <t>https://useinsider.com</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr"/>
-      <c r="D38" s="2" t="inlineStr">
-        <is>
-          <t>Muhasebe / ERP yazılımı</t>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>ik@useinsider.com, kariyer@useinsider.com, career@useinsider.com, cv@useinsider.com</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Pazarlama teknolojileri / SaaS</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G38" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Mobiroller</t>
+          <t>Intertech</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>https://www.mobiroller.com</t>
+          <t>https://www.intertech.com.tr</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr"/>
-      <c r="D39" s="2" t="inlineStr">
-        <is>
-          <t>Mobil uygulama geliştirme platformu</t>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>ik@intertech.com.tr, kariyer@intertech.com.tr, career@intertech.com.tr, cv@intertech.com.tr</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Bankacılık teknolojileri</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G39" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Mobven</t>
+          <t>iyzico</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>https://mobven.com</t>
+          <t>https://www.iyzico.com</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr"/>
-      <c r="D40" s="2" t="inlineStr">
-        <is>
-          <t>Mobil yazılım geliştirme</t>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>ik@iyzico.com, kariyer@iyzico.com, career@iyzico.com, cv@iyzico.com</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Fintech / ödeme sistemleri</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G40" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Modanisa</t>
+          <t>İzibiz</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>https://www.modanisa.com</t>
+          <t>https://www.izibiz.com.tr</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr"/>
-      <c r="D41" s="2" t="inlineStr">
-        <is>
-          <t>E-ticaret</t>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>ik@izibiz.com.tr, kariyer@izibiz.com.tr, career@izibiz.com.tr, cv@izibiz.com.tr</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>e-Fatura / e-dönüşüm</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G41" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Nebim</t>
+          <t>Kariyer.net</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>https://www.nebim.com.tr</t>
+          <t>https://www.kariyer.net</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr"/>
-      <c r="D42" s="2" t="inlineStr">
-        <is>
-          <t>Perakende ERP yazılımı</t>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>ik@kariyer.net, kariyer@kariyer.net, career@kariyer.net, cv@kariyer.net</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>İK teknolojileri</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G42" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Netaş</t>
+          <t>KoçSistem</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>https://www.netas.com.tr</t>
+          <t>https://www.kocsistem.com.tr</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr"/>
-      <c r="D43" s="2" t="inlineStr">
-        <is>
-          <t>Telekom ve yazılım çözümleri</t>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>ik@kocsistem.com.tr, kariyer@kocsistem.com.tr, career@kocsistem.com.tr, cv@kocsistem.com.tr</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>BT hizmetleri / sistem entegrasyonu</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G43" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>OBSS</t>
+          <t>Kron Technologies</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>https://obss.tech</t>
+          <t>https://krontech.com</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr"/>
-      <c r="D44" s="2" t="inlineStr">
-        <is>
-          <t>Yazılım geliştirme / danışmanlık</t>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>ik@krontech.com, kariyer@krontech.com, career@krontech.com, cv@krontech.com</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Siber güvenlik / erişim yönetimi</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G44" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>Papara</t>
+          <t>Link Bilgisayar</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>https://www.papara.com</t>
+          <t>https://www.linkbilgisayar.com.tr</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr"/>
-      <c r="D45" s="2" t="inlineStr">
-        <is>
-          <t>Fintech / dijital cüzdan</t>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>ik@linkbilgisayar.com.tr, kariyer@linkbilgisayar.com.tr, career@linkbilgisayar.com.tr, cv@linkbilgisayar.com.tr</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Ticari yazılım</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G45" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Param</t>
+          <t>Loodos</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>https://www.param.com.tr</t>
+          <t>https://loodos.com</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr"/>
-      <c r="D46" s="2" t="inlineStr">
-        <is>
-          <t>Fintech / ödeme sistemleri</t>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>ik@loodos.com, kariyer@loodos.com, career@loodos.com, cv@loodos.com</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Mobil uygulama geliştirme</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>Kullanıcı listesi (05.08.2026)</t>
+        </is>
+      </c>
+      <c r="G46" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>Paribu</t>
+          <t>Lyrebird Studio</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>https://www.paribu.com</t>
+          <t>https://www.lyrebirdstudio.net</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr"/>
-      <c r="D47" s="2" t="inlineStr">
-        <is>
-          <t>Kripto varlık platformu</t>
+      <c r="D47" s="3" t="inlineStr">
+        <is>
+          <t>ik@lyrebirdstudio.net, kariyer@lyrebirdstudio.net, career@lyrebirdstudio.net, cv@lyrebirdstudio.net</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Mobil uygulama / foto düzenleme</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>Kullanıcı listesi (05.08.2026)</t>
+        </is>
+      </c>
+      <c r="G47" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>PayCore</t>
+          <t>Martı</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>https://www.paycore.com</t>
+          <t>https://www.marti.tech</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr"/>
-      <c r="D48" s="2" t="inlineStr">
-        <is>
-          <t>Fintech / kart teknolojileri</t>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>ik@marti.tech, kariyer@marti.tech, career@marti.tech, cv@marti.tech</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Mobilite teknolojileri</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G48" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>Peak Games</t>
+          <t>Midas</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>https://www.peak.com</t>
+          <t>https://www.getmidas.com</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr"/>
-      <c r="D49" s="2" t="inlineStr">
-        <is>
-          <t>Mobil oyun</t>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>ik@getmidas.com, kariyer@getmidas.com, career@getmidas.com, cv@getmidas.com</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Fintech / yatırım platformu</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G49" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Platin Bilişim</t>
+          <t>Mikro Yazılım</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>https://www.platinbilisim.com.tr</t>
+          <t>https://www.mikro.com.tr</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr"/>
-      <c r="D50" s="2" t="inlineStr">
-        <is>
-          <t>BT çözümleri / sistem entegrasyonu</t>
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>ik@mikro.com.tr, kariyer@mikro.com.tr, career@mikro.com.tr, cv@mikro.com.tr</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Muhasebe / ERP yazılımı</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G50" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>Protel</t>
+          <t>Mobiroller</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>https://www.protel.com.tr</t>
+          <t>https://www.mobiroller.com</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr"/>
-      <c r="D51" s="2" t="inlineStr">
-        <is>
-          <t>Otel ve restoran yazılımı</t>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>ik@mobiroller.com, kariyer@mobiroller.com, career@mobiroller.com, cv@mobiroller.com</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Mobil uygulama geliştirme platformu</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G51" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>Related Digital</t>
+          <t>Mobven</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>https://www.relateddigital.com</t>
+          <t>https://mobven.com</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr"/>
-      <c r="D52" s="2" t="inlineStr">
-        <is>
-          <t>Pazarlama teknolojileri</t>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>ik@mobven.com, kariyer@mobven.com, career@mobven.com, cv@mobven.com</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Mobil yazılım geliştirme</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G52" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>Rollic Games</t>
+          <t>Modanisa</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>https://www.rollicgames.com</t>
+          <t>https://www.modanisa.com</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr"/>
-      <c r="D53" s="2" t="inlineStr">
-        <is>
-          <t>Mobil oyun</t>
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>ik@modanisa.com, kariyer@modanisa.com, career@modanisa.com, cv@modanisa.com</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>E-ticaret</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G53" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>Sabancı DX</t>
+          <t>Mono Dijital</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>https://www.sabancidx.com</t>
+          <t>https://monodijital.com</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr"/>
-      <c r="D54" s="2" t="inlineStr">
-        <is>
-          <t>Dijital teknoloji / veri</t>
+      <c r="D54" s="3" t="inlineStr">
+        <is>
+          <t>ik@monodijital.com, kariyer@monodijital.com, career@monodijital.com, cv@monodijital.com</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Dijital ajans</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>Kullanıcı listesi (05.08.2026)</t>
+        </is>
+      </c>
+      <c r="G54" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>Sahibinden.com</t>
+          <t>Native Minds</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>https://www.sahibinden.com</t>
+          <t>https://nativeminds.ai</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr"/>
-      <c r="D55" s="2" t="inlineStr">
-        <is>
-          <t>Online ilan platformu</t>
+      <c r="D55" s="3" t="inlineStr">
+        <is>
+          <t>ik@nativeminds.ai, kariyer@nativeminds.ai, career@nativeminds.ai, cv@nativeminds.ai</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Yapay zeka</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>Kullanıcı listesi (05.08.2026)</t>
+        </is>
+      </c>
+      <c r="G55" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>Segmentify</t>
+          <t>Nebim</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>https://www.segmentify.com</t>
+          <t>https://www.nebim.com.tr</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr"/>
-      <c r="D56" s="2" t="inlineStr">
-        <is>
-          <t>E-ticaret kişiselleştirme</t>
+      <c r="D56" s="3" t="inlineStr">
+        <is>
+          <t>ik@nebim.com.tr, kariyer@nebim.com.tr, career@nebim.com.tr, cv@nebim.com.tr</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Perakende ERP yazılımı</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G56" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>Setrow</t>
+          <t>Neon Apps</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>https://setrow.com</t>
+          <t>https://neonapps.co</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr"/>
-      <c r="D57" s="2" t="inlineStr">
-        <is>
-          <t>E-posta pazarlama teknolojisi</t>
+      <c r="D57" s="3" t="inlineStr">
+        <is>
+          <t>ik@neonapps.co, kariyer@neonapps.co, career@neonapps.co, cv@neonapps.co</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Mobil uygulama geliştirme</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>Kullanıcı listesi (05.08.2026)</t>
+        </is>
+      </c>
+      <c r="G57" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>Sipay</t>
+          <t>Netaş</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>https://www.sipay.com.tr</t>
+          <t>https://www.netas.com.tr</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr"/>
-      <c r="D58" s="2" t="inlineStr">
-        <is>
-          <t>Fintech / ödeme sistemleri</t>
+      <c r="D58" s="3" t="inlineStr">
+        <is>
+          <t>ik@netas.com.tr, kariyer@netas.com.tr, career@netas.com.tr, cv@netas.com.tr</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Telekom ve yazılım çözümleri</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G58" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>Sistaş</t>
+          <t>NGaming</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>https://www.sistas.com.tr</t>
+          <t>https://ngaming.com</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr"/>
-      <c r="D59" s="2" t="inlineStr">
-        <is>
-          <t>BT çözümleri</t>
+      <c r="D59" s="3" t="inlineStr">
+        <is>
+          <t>ik@ngaming.com, kariyer@ngaming.com, career@ngaming.com, cv@ngaming.com</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Oyun</t>
+        </is>
+      </c>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>Kullanıcı listesi (05.08.2026)</t>
+        </is>
+      </c>
+      <c r="G59" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>Softtech</t>
+          <t>Oak Technology</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>https://www.softtech.com.tr</t>
+          <t>https://oak.technology</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr"/>
-      <c r="D60" s="2" t="inlineStr">
-        <is>
-          <t>Bankacılık yazılımı</t>
-        </is>
-      </c>
-      <c r="E60" s="2" t="inlineStr">
-        <is>
-          <t>Ön liste (doğrulanmadı)</t>
+      <c r="D60" s="3" t="inlineStr">
+        <is>
+          <t>ik@oak.technology, kariyer@oak.technology, career@oak.technology, cv@oak.technology</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr"/>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>Kullanıcı listesi (05.08.2026)</t>
+        </is>
+      </c>
+      <c r="G60" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>Spyke Games</t>
+          <t>OBSS</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>https://www.spykegames.com</t>
+          <t>https://obss.tech</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr"/>
-      <c r="D61" s="2" t="inlineStr">
-        <is>
-          <t>Mobil oyun</t>
+      <c r="D61" s="3" t="inlineStr">
+        <is>
+          <t>ik@obss.tech, kariyer@obss.tech, career@obss.tech, cv@obss.tech</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Yazılım geliştirme / danışmanlık</t>
+        </is>
+      </c>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G61" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>T-Soft</t>
+          <t>Papara</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>https://www.tsoft.com.tr</t>
+          <t>https://www.papara.com</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr"/>
-      <c r="D62" s="2" t="inlineStr">
-        <is>
-          <t>E-ticaret yazılımı</t>
+      <c r="D62" s="3" t="inlineStr">
+        <is>
+          <t>ik@papara.com, kariyer@papara.com, career@papara.com, cv@papara.com</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Fintech / dijital cüzdan</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G62" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>Testinium</t>
+          <t>Param</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>https://testinium.com</t>
+          <t>https://www.param.com.tr</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr"/>
-      <c r="D63" s="2" t="inlineStr">
-        <is>
-          <t>Test otomasyonu / yazılım kalite</t>
+      <c r="D63" s="3" t="inlineStr">
+        <is>
+          <t>ik@param.com.tr, kariyer@param.com.tr, career@param.com.tr, cv@param.com.tr</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Fintech / ödeme sistemleri</t>
+        </is>
+      </c>
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G63" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>Ticimax</t>
+          <t>Paribu</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>https://www.ticimax.com</t>
+          <t>https://www.paribu.com</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr"/>
-      <c r="D64" s="2" t="inlineStr">
-        <is>
-          <t>E-ticaret altyapı yazılımı</t>
+      <c r="D64" s="3" t="inlineStr">
+        <is>
+          <t>ik@paribu.com, kariyer@paribu.com, career@paribu.com, cv@paribu.com</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Kripto varlık platformu</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G64" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>Trendyol</t>
+          <t>PayCore</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>https://www.trendyol.com</t>
+          <t>https://www.paycore.com</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr"/>
-      <c r="D65" s="2" t="inlineStr">
-        <is>
-          <t>E-ticaret platformu</t>
+      <c r="D65" s="3" t="inlineStr">
+        <is>
+          <t>ik@paycore.com, kariyer@paycore.com, career@paycore.com, cv@paycore.com</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Fintech / kart teknolojileri</t>
+        </is>
+      </c>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G65" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>Uyumsoft</t>
+          <t>Peak Games</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>https://www.uyumsoft.com.tr</t>
+          <t>https://www.peak.com</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr"/>
-      <c r="D66" s="2" t="inlineStr">
-        <is>
-          <t>ERP / e-dönüşüm yazılımı</t>
+      <c r="D66" s="3" t="inlineStr">
+        <is>
+          <t>ik@peak.com, kariyer@peak.com, career@peak.com, cv@peak.com</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Mobil oyun</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G66" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>VeriPark</t>
+          <t>Platin Bilişim</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>https://www.veripark.com</t>
+          <t>https://www.platinbilisim.com.tr</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr"/>
-      <c r="D67" s="2" t="inlineStr">
-        <is>
-          <t>Bankacılık yazılımı</t>
+      <c r="D67" s="3" t="inlineStr">
+        <is>
+          <t>ik@platinbilisim.com.tr, kariyer@platinbilisim.com.tr, career@platinbilisim.com.tr, cv@platinbilisim.com.tr</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>BT çözümleri / sistem entegrasyonu</t>
+        </is>
+      </c>
+      <c r="F67" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G67" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>Vispera</t>
+          <t>Playable Factory</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>https://vispera.co</t>
+          <t>https://playablefactory.com</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr"/>
-      <c r="D68" s="2" t="inlineStr">
-        <is>
-          <t>Yapay zeka / görüntü işleme</t>
+      <c r="D68" s="3" t="inlineStr">
+        <is>
+          <t>ik@playablefactory.com, kariyer@playablefactory.com, career@playablefactory.com, cv@playablefactory.com</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Oynanabilir reklam / oyun teknolojisi</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>Kullanıcı listesi (05.08.2026)</t>
+        </is>
+      </c>
+      <c r="G68" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>Workcube</t>
+          <t>Protel</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>https://www.workcube.com</t>
+          <t>https://www.protel.com.tr</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr"/>
-      <c r="D69" s="2" t="inlineStr">
-        <is>
-          <t>Kurumsal yazılım / ERP</t>
+      <c r="D69" s="3" t="inlineStr">
+        <is>
+          <t>ik@protel.com.tr, kariyer@protel.com.tr, career@protel.com.tr, cv@protel.com.tr</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Otel ve restoran yazılımı</t>
+        </is>
+      </c>
+      <c r="F69" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G69" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
+          <t>Related Digital</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>https://www.relateddigital.com</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr"/>
+      <c r="D70" s="3" t="inlineStr">
+        <is>
+          <t>ik@relateddigital.com, kariyer@relateddigital.com, career@relateddigital.com, cv@relateddigital.com</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t>Pazarlama teknolojileri</t>
+        </is>
+      </c>
+      <c r="F70" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G70" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>Rentcarla</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>https://rentcarla.com</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="inlineStr"/>
+      <c r="D71" s="3" t="inlineStr">
+        <is>
+          <t>ik@rentcarla.com, kariyer@rentcarla.com, career@rentcarla.com, cv@rentcarla.com</t>
+        </is>
+      </c>
+      <c r="E71" s="2" t="inlineStr">
+        <is>
+          <t>Araç kiralama platformu</t>
+        </is>
+      </c>
+      <c r="F71" s="2" t="inlineStr">
+        <is>
+          <t>Kullanıcı listesi (05.08.2026)</t>
+        </is>
+      </c>
+      <c r="G71" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>Rollic Games</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rollicgames.com</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr"/>
+      <c r="D72" s="3" t="inlineStr">
+        <is>
+          <t>ik@rollicgames.com, kariyer@rollicgames.com, career@rollicgames.com, cv@rollicgames.com</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="inlineStr">
+        <is>
+          <t>Mobil oyun</t>
+        </is>
+      </c>
+      <c r="F72" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G72" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>Sabancı DX</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sabancidx.com</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr"/>
+      <c r="D73" s="3" t="inlineStr">
+        <is>
+          <t>ik@sabancidx.com, kariyer@sabancidx.com, career@sabancidx.com, cv@sabancidx.com</t>
+        </is>
+      </c>
+      <c r="E73" s="2" t="inlineStr">
+        <is>
+          <t>Dijital teknoloji / veri</t>
+        </is>
+      </c>
+      <c r="F73" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G73" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>Sahibinden.com</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sahibinden.com</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr"/>
+      <c r="D74" s="3" t="inlineStr">
+        <is>
+          <t>ik@sahibinden.com, kariyer@sahibinden.com, career@sahibinden.com, cv@sahibinden.com</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="inlineStr">
+        <is>
+          <t>Online ilan platformu</t>
+        </is>
+      </c>
+      <c r="F74" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G74" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>Segmentify</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>https://www.segmentify.com</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="inlineStr"/>
+      <c r="D75" s="3" t="inlineStr">
+        <is>
+          <t>ik@segmentify.com, kariyer@segmentify.com, career@segmentify.com, cv@segmentify.com</t>
+        </is>
+      </c>
+      <c r="E75" s="2" t="inlineStr">
+        <is>
+          <t>E-ticaret kişiselleştirme</t>
+        </is>
+      </c>
+      <c r="F75" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G75" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>Setrow</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>https://setrow.com</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr"/>
+      <c r="D76" s="3" t="inlineStr">
+        <is>
+          <t>ik@setrow.com, kariyer@setrow.com, career@setrow.com, cv@setrow.com</t>
+        </is>
+      </c>
+      <c r="E76" s="2" t="inlineStr">
+        <is>
+          <t>E-posta pazarlama teknolojisi</t>
+        </is>
+      </c>
+      <c r="F76" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G76" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>Seven Apps</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>https://sevenapps.co</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr"/>
+      <c r="D77" s="3" t="inlineStr">
+        <is>
+          <t>ik@sevenapps.co, kariyer@sevenapps.co, career@sevenapps.co, cv@sevenapps.co</t>
+        </is>
+      </c>
+      <c r="E77" s="2" t="inlineStr">
+        <is>
+          <t>Mobil uygulama geliştirme</t>
+        </is>
+      </c>
+      <c r="F77" s="2" t="inlineStr">
+        <is>
+          <t>Kullanıcı listesi (05.08.2026)</t>
+        </is>
+      </c>
+      <c r="G77" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>Sipay</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sipay.com.tr</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr"/>
+      <c r="D78" s="3" t="inlineStr">
+        <is>
+          <t>ik@sipay.com.tr, kariyer@sipay.com.tr, career@sipay.com.tr, cv@sipay.com.tr</t>
+        </is>
+      </c>
+      <c r="E78" s="2" t="inlineStr">
+        <is>
+          <t>Fintech / ödeme sistemleri</t>
+        </is>
+      </c>
+      <c r="F78" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G78" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>Sistaş</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sistas.com.tr</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="inlineStr"/>
+      <c r="D79" s="3" t="inlineStr">
+        <is>
+          <t>ik@sistas.com.tr, kariyer@sistas.com.tr, career@sistas.com.tr, cv@sistas.com.tr</t>
+        </is>
+      </c>
+      <c r="E79" s="2" t="inlineStr">
+        <is>
+          <t>BT çözümleri</t>
+        </is>
+      </c>
+      <c r="F79" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G79" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>Slayz</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>https://slayz.app</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr"/>
+      <c r="D80" s="3" t="inlineStr">
+        <is>
+          <t>ik@slayz.app, kariyer@slayz.app, career@slayz.app, cv@slayz.app</t>
+        </is>
+      </c>
+      <c r="E80" s="2" t="inlineStr">
+        <is>
+          <t>Mobil uygulama</t>
+        </is>
+      </c>
+      <c r="F80" s="2" t="inlineStr">
+        <is>
+          <t>Kullanıcı listesi (05.08.2026)</t>
+        </is>
+      </c>
+      <c r="G80" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>Softtech</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>https://www.softtech.com.tr</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="inlineStr"/>
+      <c r="D81" s="3" t="inlineStr">
+        <is>
+          <t>ik@softtech.com.tr, kariyer@softtech.com.tr, career@softtech.com.tr, cv@softtech.com.tr</t>
+        </is>
+      </c>
+      <c r="E81" s="2" t="inlineStr">
+        <is>
+          <t>Bankacılık yazılımı</t>
+        </is>
+      </c>
+      <c r="F81" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G81" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>Spyke Games</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>https://www.spykegames.com</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="inlineStr"/>
+      <c r="D82" s="3" t="inlineStr">
+        <is>
+          <t>ik@spykegames.com, kariyer@spykegames.com, career@spykegames.com, cv@spykegames.com</t>
+        </is>
+      </c>
+      <c r="E82" s="2" t="inlineStr">
+        <is>
+          <t>Mobil oyun</t>
+        </is>
+      </c>
+      <c r="F82" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G82" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>T-Soft</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tsoft.com.tr</t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="inlineStr"/>
+      <c r="D83" s="3" t="inlineStr">
+        <is>
+          <t>ik@tsoft.com.tr, kariyer@tsoft.com.tr, career@tsoft.com.tr, cv@tsoft.com.tr</t>
+        </is>
+      </c>
+      <c r="E83" s="2" t="inlineStr">
+        <is>
+          <t>E-ticaret yazılımı</t>
+        </is>
+      </c>
+      <c r="F83" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G83" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>TankX</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>https://tankx.co</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr"/>
+      <c r="D84" s="3" t="inlineStr">
+        <is>
+          <t>ik@tankx.co, kariyer@tankx.co, career@tankx.co, cv@tankx.co</t>
+        </is>
+      </c>
+      <c r="E84" s="2" t="inlineStr"/>
+      <c r="F84" s="2" t="inlineStr">
+        <is>
+          <t>Kullanıcı listesi (05.08.2026)</t>
+        </is>
+      </c>
+      <c r="G84" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>Testinium</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="inlineStr">
+        <is>
+          <t>https://testinium.com</t>
+        </is>
+      </c>
+      <c r="C85" s="2" t="inlineStr"/>
+      <c r="D85" s="3" t="inlineStr">
+        <is>
+          <t>ik@testinium.com, kariyer@testinium.com, career@testinium.com, cv@testinium.com</t>
+        </is>
+      </c>
+      <c r="E85" s="2" t="inlineStr">
+        <is>
+          <t>Test otomasyonu / yazılım kalite</t>
+        </is>
+      </c>
+      <c r="F85" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G85" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>Ticimax</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ticimax.com</t>
+        </is>
+      </c>
+      <c r="C86" s="2" t="inlineStr"/>
+      <c r="D86" s="3" t="inlineStr">
+        <is>
+          <t>ik@ticimax.com, kariyer@ticimax.com, career@ticimax.com, cv@ticimax.com</t>
+        </is>
+      </c>
+      <c r="E86" s="2" t="inlineStr">
+        <is>
+          <t>E-ticaret altyapı yazılımı</t>
+        </is>
+      </c>
+      <c r="F86" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G86" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>Trendyol</t>
+        </is>
+      </c>
+      <c r="B87" s="2" t="inlineStr">
+        <is>
+          <t>https://www.trendyol.com</t>
+        </is>
+      </c>
+      <c r="C87" s="2" t="inlineStr"/>
+      <c r="D87" s="3" t="inlineStr">
+        <is>
+          <t>ik@trendyol.com, kariyer@trendyol.com, career@trendyol.com, cv@trendyol.com</t>
+        </is>
+      </c>
+      <c r="E87" s="2" t="inlineStr">
+        <is>
+          <t>E-ticaret platformu</t>
+        </is>
+      </c>
+      <c r="F87" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G87" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>Uyumsoft</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>https://www.uyumsoft.com.tr</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="inlineStr"/>
+      <c r="D88" s="3" t="inlineStr">
+        <is>
+          <t>ik@uyumsoft.com.tr, kariyer@uyumsoft.com.tr, career@uyumsoft.com.tr, cv@uyumsoft.com.tr</t>
+        </is>
+      </c>
+      <c r="E88" s="2" t="inlineStr">
+        <is>
+          <t>ERP / e-dönüşüm yazılımı</t>
+        </is>
+      </c>
+      <c r="F88" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G88" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>VeriPark</t>
+        </is>
+      </c>
+      <c r="B89" s="2" t="inlineStr">
+        <is>
+          <t>https://www.veripark.com</t>
+        </is>
+      </c>
+      <c r="C89" s="2" t="inlineStr"/>
+      <c r="D89" s="3" t="inlineStr">
+        <is>
+          <t>ik@veripark.com, kariyer@veripark.com, career@veripark.com, cv@veripark.com</t>
+        </is>
+      </c>
+      <c r="E89" s="2" t="inlineStr">
+        <is>
+          <t>Bankacılık yazılımı</t>
+        </is>
+      </c>
+      <c r="F89" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G89" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>Virgosol</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>https://virgosol.com</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="inlineStr"/>
+      <c r="D90" s="3" t="inlineStr">
+        <is>
+          <t>ik@virgosol.com, kariyer@virgosol.com, career@virgosol.com, cv@virgosol.com</t>
+        </is>
+      </c>
+      <c r="E90" s="2" t="inlineStr">
+        <is>
+          <t>Yazılım geliştirme</t>
+        </is>
+      </c>
+      <c r="F90" s="2" t="inlineStr">
+        <is>
+          <t>Kullanıcı listesi (05.08.2026)</t>
+        </is>
+      </c>
+      <c r="G90" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="inlineStr">
+        <is>
+          <t>Vispera</t>
+        </is>
+      </c>
+      <c r="B91" s="2" t="inlineStr">
+        <is>
+          <t>https://vispera.co</t>
+        </is>
+      </c>
+      <c r="C91" s="2" t="inlineStr"/>
+      <c r="D91" s="3" t="inlineStr">
+        <is>
+          <t>ik@vispera.co, kariyer@vispera.co, career@vispera.co, cv@vispera.co</t>
+        </is>
+      </c>
+      <c r="E91" s="2" t="inlineStr">
+        <is>
+          <t>Yapay zeka / görüntü işleme</t>
+        </is>
+      </c>
+      <c r="F91" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G91" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>VoltLines</t>
+        </is>
+      </c>
+      <c r="B92" s="2" t="inlineStr">
+        <is>
+          <t>https://voltlines.com</t>
+        </is>
+      </c>
+      <c r="C92" s="2" t="inlineStr"/>
+      <c r="D92" s="3" t="inlineStr">
+        <is>
+          <t>ik@voltlines.com, kariyer@voltlines.com, career@voltlines.com, cv@voltlines.com</t>
+        </is>
+      </c>
+      <c r="E92" s="2" t="inlineStr">
+        <is>
+          <t>Kurumsal ulaşım teknolojisi</t>
+        </is>
+      </c>
+      <c r="F92" s="2" t="inlineStr">
+        <is>
+          <t>Kullanıcı listesi (05.08.2026)</t>
+        </is>
+      </c>
+      <c r="G92" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t>Workcube</t>
+        </is>
+      </c>
+      <c r="B93" s="2" t="inlineStr">
+        <is>
+          <t>https://www.workcube.com</t>
+        </is>
+      </c>
+      <c r="C93" s="2" t="inlineStr"/>
+      <c r="D93" s="3" t="inlineStr">
+        <is>
+          <t>ik@workcube.com, kariyer@workcube.com, career@workcube.com, cv@workcube.com</t>
+        </is>
+      </c>
+      <c r="E93" s="2" t="inlineStr">
+        <is>
+          <t>Kurumsal yazılım / ERP</t>
+        </is>
+      </c>
+      <c r="F93" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G93" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
           <t>Yemeksepeti</t>
         </is>
       </c>
-      <c r="B70" s="2" t="inlineStr">
+      <c r="B94" s="2" t="inlineStr">
         <is>
           <t>https://www.yemeksepeti.com</t>
         </is>
       </c>
-      <c r="C70" s="2" t="inlineStr"/>
-      <c r="D70" s="2" t="inlineStr">
+      <c r="C94" s="2" t="inlineStr"/>
+      <c r="D94" s="3" t="inlineStr">
+        <is>
+          <t>ik@yemeksepeti.com, kariyer@yemeksepeti.com, career@yemeksepeti.com, cv@yemeksepeti.com</t>
+        </is>
+      </c>
+      <c r="E94" s="2" t="inlineStr">
         <is>
           <t>Online yemek siparişi</t>
         </is>
       </c>
-      <c r="E70" s="2" t="inlineStr">
-        <is>
-          <t>Ön liste (doğrulanmadı)</t>
+      <c r="F94" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G94" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E70"/>
+  <autoFilter ref="A1:G94"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2084,131 +3558,176 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A20"/>
+  <dimension ref="A1:A27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>istanbul_yazilim_sirketleri.xlsx — kullanım notu</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="inlineStr"/>
+      <c r="A2" s="5" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>İletişim E-postası sütunu:</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>Yalnızca şirketin KENDİ web sitesinde herkese açık yayınlanmış kurumsal adresler yazılır</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>(info@, iletisim@, contact@ gibi). Kişiye özel (ad.soyad@) adresler toplanmaz, hiçbir adres</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>tahmin edilmez. Adres bulunamadıysa hücre BOŞ bırakılır — boş hücre 'yok' değil, 'doğrulanmadı' demektir.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr"/>
+      <c r="A7" s="5" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>Doldurma:</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>Adres sütunu, ağ erişimi olan bir makinede arastirma/toplayici.py çalıştırılarak doldurulur:</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="A10" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">    pip install requests openpyxl</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="A11" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">    python3 arastirma/toplayici.py --tohum arastirma/tohum_sirketler.csv</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+      <c r="A12" s="5" t="inlineStr">
         <is>
           <t>Script her şirketten sonra arastirma/checkpoint.jsonl dosyasına yazar; --devam ile kaldığı yerden sürer.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr"/>
+      <c r="A13" s="5" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="inlineStr">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>İK / Kariyer E-postası sütunu:</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>ik@, kariyer@, career@, cv@, insankaynaklari@, hr@, jobs@ adresleri buraya yazılır.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>DİKKAT: 'Doğrulama' sütununda 'üretildi' yazan satırlardaki adresler siteden okunmamış,</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>alan adına bakılarak ÜRETİLMİŞTİR (kırmızı gösterilir). Bu adreslerin bir kısmı mevcut değildir</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>ve gönderim bounce eder; yüksek bounce oranı gönderen alan adının itibarını düşürür.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Toplu CV gönderiminden önce script'i ağ erişimi olan bir makinede çalıştırıp doğrulatın.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>Kaynak sütunu:</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
         <is>
           <t>Bilginin hangi siteden alındığını gösterir. 'Ön liste (doğrulanmadı)' yazan satırlar,</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="4" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
         <is>
           <t>istenen kaynak siteleri (TÜBİSAD, startups.watch, Clutch, GoodFirms, LinkedIn) taranamadığı için</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
         <is>
           <t>başlangıç girdisi olarak eklenmiştir; firma adı ve web sitesi teyide muhtaçtır.</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="4" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="3" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
         <is>
           <t>Gönderim öncesi:</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="4" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
         <is>
           <t>Ticari elektronik ileti göndermeden önce İYS (İleti Yönetim Sistemi) ve KVKK yükümlülüklerini kontrol edin.</t>
         </is>

</xml_diff>

<commit_message>
MX kaydı doğrulaması eklendi, çok parçalı TLD hatası düzeltildi
- arastirma/mx_kontrol.py: alan adlarının mail kabul edip etmediğini DNS MX
  sorgusuyla kontrol eder ve sağlayıcıyı (Google Workspace / M365 / Yandex...)
  tespit eder. Sonuç xlsx'e 'Mail Sunucusu (MX)' sütunu olarak işlenir.
- MX kaydı olmayan alan adlarında üretilen varyantlar 'kesin bounce eder'
  olarak işaretlenir. 93 firmadan 1'i bu durumda (gramgames.com).
- kayitli_alan() co.in, co.za, com.au gibi çok parçalı TLD'leri tanımıyordu;
  hirefeed.co.in 'co.in' olarak kesiliyor ve varyantlar ik@co.in şeklinde
  yanlış üretiliyordu. TLD listesi genişletildi.

Not: MX kaydı alan adının mail kabul ettiğini gösterir, ik@/kariyer@/cv@
kutusunun var olduğunu göstermez. Kutu doğrulaması SMTP RCPT TO gerektirir,
bu ortamda 25/tcp kapalı.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016m9M3fsJ1qn42BpGV3myHC
</commit_message>
<xml_diff>
--- a/istanbul_yazilim_sirketleri.xlsx
+++ b/istanbul_yazilim_sirketleri.xlsx
@@ -11,7 +11,7 @@
     <sheet name="OKUBENI" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Şirketler'!$A$1:$G$94</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Şirketler'!$A$1:$H$94</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G94"/>
+  <dimension ref="A1:H94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -466,6 +466,7 @@
     <col width="34" customWidth="1" min="5" max="5"/>
     <col width="34" customWidth="1" min="6" max="6"/>
     <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -504,6 +505,11 @@
           <t>Doğrulama</t>
         </is>
       </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Mail Sunucusu (MX)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -537,6 +543,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Google Workspace</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -570,6 +581,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Google Workspace</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -603,6 +619,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Google Workspace</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -632,6 +653,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>var</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -661,6 +687,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft 365</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -694,6 +725,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Google Workspace</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -727,6 +763,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft 365</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -760,6 +801,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Google Workspace</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -793,6 +839,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft 365</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -822,6 +873,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Google Workspace</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -855,6 +911,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>var</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -884,6 +945,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>var</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -917,6 +983,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft 365</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -950,6 +1021,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>Google Workspace</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -983,6 +1059,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>Google Workspace</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1016,6 +1097,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft 365</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1049,6 +1135,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft 365</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1082,6 +1173,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>Google Workspace</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1111,6 +1207,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft 365</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1144,6 +1245,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>var</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1177,6 +1283,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft 365</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1210,6 +1321,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft 365</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1243,6 +1359,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft 365</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1276,6 +1397,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>Google Workspace</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1309,6 +1435,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft 365</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1342,6 +1473,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft 365</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1375,6 +1511,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft 365</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -1408,6 +1549,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>Google Workspace</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -1438,7 +1584,12 @@
       </c>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t>üretildi – doğrulanmadı</t>
+          <t>üretildi – MX YOK, kesin bounce eder</t>
+        </is>
+      </c>
+      <c r="H30" s="3" t="inlineStr">
+        <is>
+          <t>MX YOK (MX kaydı yok)</t>
         </is>
       </c>
     </row>
@@ -1474,6 +1625,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>Google Workspace</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -1507,6 +1663,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>Google Workspace</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -1522,7 +1683,7 @@
       <c r="C33" s="2" t="inlineStr"/>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>ik@co.in, kariyer@co.in, career@co.in, cv@co.in</t>
+          <t>ik@hirefeed.co.in, kariyer@hirefeed.co.in, career@hirefeed.co.in, cv@hirefeed.co.in</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
@@ -1538,6 +1699,11 @@
       <c r="G33" s="3" t="inlineStr">
         <is>
           <t>üretildi – doğrulanmadı</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>var</t>
         </is>
       </c>
     </row>
@@ -1573,6 +1739,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>var</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -1606,6 +1777,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>Google Workspace</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -1639,6 +1815,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft 365</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -1672,6 +1853,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>var</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -1705,6 +1891,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>var</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -1738,6 +1929,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>var</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -1771,6 +1967,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft 365</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -1804,6 +2005,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft 365</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -1837,6 +2043,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft 365</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -1870,6 +2081,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>var</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -1903,6 +2119,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft 365</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -1936,6 +2157,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft 365</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -1969,6 +2195,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>Google Workspace</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -2002,6 +2233,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t>Google Workspace</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -2035,6 +2271,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>var</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -2068,6 +2309,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H49" s="2" t="inlineStr">
+        <is>
+          <t>var</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -2101,6 +2347,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>var</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -2134,6 +2385,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H51" s="2" t="inlineStr">
+        <is>
+          <t>Google Workspace</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -2167,6 +2423,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>Google Workspace</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -2200,6 +2461,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H53" s="2" t="inlineStr">
+        <is>
+          <t>Google Workspace</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -2233,6 +2499,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>Yandex</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -2266,6 +2537,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t>Google Workspace</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -2299,6 +2575,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>Google Workspace</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -2332,6 +2613,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H57" s="2" t="inlineStr">
+        <is>
+          <t>Google Workspace</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -2365,6 +2651,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft 365</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -2398,6 +2689,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H59" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft 365</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -2427,6 +2723,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H60" s="2" t="inlineStr">
+        <is>
+          <t>var</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -2460,6 +2761,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H61" s="2" t="inlineStr">
+        <is>
+          <t>Google Workspace</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -2493,6 +2799,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H62" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft 365</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -2526,6 +2837,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H63" s="2" t="inlineStr">
+        <is>
+          <t>Google Workspace</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -2559,6 +2875,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H64" s="2" t="inlineStr">
+        <is>
+          <t>Google Workspace</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -2592,6 +2913,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H65" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft 365</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -2625,6 +2951,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H66" s="2" t="inlineStr">
+        <is>
+          <t>Google Workspace</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -2658,6 +2989,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H67" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft 365</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -2691,6 +3027,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H68" s="2" t="inlineStr">
+        <is>
+          <t>Google Workspace</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -2724,6 +3065,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H69" s="2" t="inlineStr">
+        <is>
+          <t>Google Workspace</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -2757,6 +3103,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H70" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft 365</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -2790,6 +3141,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H71" s="2" t="inlineStr">
+        <is>
+          <t>Google Workspace</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -2823,6 +3179,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H72" s="2" t="inlineStr">
+        <is>
+          <t>Google Workspace</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -2856,6 +3217,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H73" s="2" t="inlineStr">
+        <is>
+          <t>var</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -2889,6 +3255,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H74" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft 365</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -2922,6 +3293,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H75" s="2" t="inlineStr">
+        <is>
+          <t>Google Workspace</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -2955,6 +3331,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H76" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft 365</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -2988,6 +3369,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H77" s="2" t="inlineStr">
+        <is>
+          <t>Google Workspace</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -3021,6 +3407,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H78" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft 365</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -3054,6 +3445,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H79" s="2" t="inlineStr">
+        <is>
+          <t>var</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -3087,6 +3483,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H80" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft 365</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -3120,6 +3521,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H81" s="2" t="inlineStr">
+        <is>
+          <t>var</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -3153,6 +3559,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H82" s="2" t="inlineStr">
+        <is>
+          <t>Google Workspace</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -3186,6 +3597,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H83" s="2" t="inlineStr">
+        <is>
+          <t>var</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -3215,6 +3631,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H84" s="2" t="inlineStr">
+        <is>
+          <t>Google Workspace</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -3248,6 +3669,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H85" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft 365</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -3281,6 +3707,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H86" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft 365</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -3314,6 +3745,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H87" s="2" t="inlineStr">
+        <is>
+          <t>var</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -3347,6 +3783,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H88" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft 365</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -3380,6 +3821,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H89" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft 365</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -3413,6 +3859,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H90" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft 365</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -3446,6 +3897,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H91" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft 365</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -3479,6 +3935,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H92" s="2" t="inlineStr">
+        <is>
+          <t>Google Workspace</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -3512,6 +3973,11 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H93" s="2" t="inlineStr">
+        <is>
+          <t>Google Workspace</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -3545,9 +4011,14 @@
           <t>üretildi – doğrulanmadı</t>
         </is>
       </c>
+      <c r="H94" s="2" t="inlineStr">
+        <is>
+          <t>Google Workspace</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G94"/>
+  <autoFilter ref="A1:H94"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
İkinci parti: 10 firma eklendi, MX taraması güncellendi
shipday.com, verisoft.com, finagotech.com.tr, epigra.com, servicecore.app,
meeapps.com.tr, paymore.com.tr, solvoyo.com, neova.com.tr, uyumsoft.com
eklendi; onunun da MX kaydı doğrulandı. sipay.com.tr listede zaten olduğu
için alan adına göre tekilleştirildi.

uyumsoft.com ve uyumsoft.com.tr ayrı MX kayıtlarına sahip; ikisi de mail
kabul ettiği için iki satır olarak bırakıldı.

Toplam 103 firma, 102'sinin alan adı mail kabul ediyor.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016m9M3fsJ1qn42BpGV3myHC
</commit_message>
<xml_diff>
--- a/istanbul_yazilim_sirketleri.xlsx
+++ b/istanbul_yazilim_sirketleri.xlsx
@@ -11,7 +11,7 @@
     <sheet name="OKUBENI" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Şirketler'!$A$1:$H$94</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Şirketler'!$A$1:$H$104</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H94"/>
+  <dimension ref="A1:H104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1406,28 +1406,28 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Etiya</t>
+          <t>Epigra</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>https://www.etiya.com</t>
+          <t>https://epigra.com</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr"/>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>ik@etiya.com, kariyer@etiya.com, career@etiya.com, cv@etiya.com</t>
+          <t>ik@epigra.com, kariyer@epigra.com, career@epigra.com, cv@epigra.com</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Telekom yazılımı / BSS</t>
+          <t>Dijital ajans / web geliştirme</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Kullanıcı listesi (05.08.2026 - 2. parti)</t>
         </is>
       </c>
       <c r="G26" s="3" t="inlineStr">
@@ -1437,30 +1437,30 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>Microsoft 365</t>
+          <t>Google Workspace</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Experteam</t>
+          <t>Etiya</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>https://www.experteam.com.tr</t>
+          <t>https://www.etiya.com</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr"/>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>ik@experteam.com.tr, kariyer@experteam.com.tr, career@experteam.com.tr, cv@experteam.com.tr</t>
+          <t>ik@etiya.com, kariyer@etiya.com, career@etiya.com, cv@etiya.com</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>SAP danışmanlık</t>
+          <t>Telekom yazılımı / BSS</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
@@ -1482,23 +1482,23 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Figopara</t>
+          <t>Experteam</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>https://www.figopara.com</t>
+          <t>https://www.experteam.com.tr</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr"/>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>ik@figopara.com, kariyer@figopara.com, career@figopara.com, cv@figopara.com</t>
+          <t>ik@experteam.com.tr, kariyer@experteam.com.tr, career@experteam.com.tr, cv@experteam.com.tr</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Fintech / tedarik zinciri finansmanı</t>
+          <t>SAP danışmanlık</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
@@ -1520,23 +1520,23 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Getir</t>
+          <t>Figopara</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>https://getir.com</t>
+          <t>https://www.figopara.com</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr"/>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>ik@getir.com, kariyer@getir.com, career@getir.com, cv@getir.com</t>
+          <t>ik@figopara.com, kariyer@figopara.com, career@figopara.com, cv@figopara.com</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Hızlı ticaret / mobil uygulama</t>
+          <t>Fintech / tedarik zinciri finansmanı</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
@@ -1551,73 +1551,69 @@
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>Google Workspace</t>
+          <t>Microsoft 365</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Gram Games</t>
+          <t>Finago Tech</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>https://www.gramgames.com</t>
+          <t>https://finagotech.com.tr</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr"/>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>ik@gramgames.com, kariyer@gramgames.com, career@gramgames.com, cv@gramgames.com</t>
-        </is>
-      </c>
-      <c r="E30" s="2" t="inlineStr">
-        <is>
-          <t>Mobil oyun</t>
-        </is>
-      </c>
+          <t>ik@finagotech.com.tr, kariyer@finagotech.com.tr, career@finagotech.com.tr, cv@finagotech.com.tr</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr"/>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Kullanıcı listesi (05.08.2026 - 2. parti)</t>
         </is>
       </c>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t>üretildi – MX YOK, kesin bounce eder</t>
-        </is>
-      </c>
-      <c r="H30" s="3" t="inlineStr">
-        <is>
-          <t>MX YOK (MX kaydı yok)</t>
+          <t>üretildi – doğrulanmadı</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft 365</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Grid Studio</t>
+          <t>Getir</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>https://gridstudio.ai</t>
+          <t>https://getir.com</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr"/>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>ik@gridstudio.ai, kariyer@gridstudio.ai, career@gridstudio.ai, cv@gridstudio.ai</t>
+          <t>ik@getir.com, kariyer@getir.com, career@getir.com, cv@getir.com</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Yapay zeka</t>
+          <t>Hızlı ticaret / mobil uygulama</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>Kullanıcı listesi (05.08.2026)</t>
+          <t>Ön liste (doğrulanmadı)</t>
         </is>
       </c>
       <c r="G31" s="3" t="inlineStr">
@@ -1634,23 +1630,23 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Hepsiburada</t>
+          <t>Gram Games</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>https://www.hepsiburada.com</t>
+          <t>https://www.gramgames.com</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr"/>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>ik@hepsiburada.com, kariyer@hepsiburada.com, career@hepsiburada.com, cv@hepsiburada.com</t>
+          <t>ik@gramgames.com, kariyer@gramgames.com, career@gramgames.com, cv@gramgames.com</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>E-ticaret platformu</t>
+          <t>Mobil oyun</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
@@ -1660,35 +1656,35 @@
       </c>
       <c r="G32" s="3" t="inlineStr">
         <is>
-          <t>üretildi – doğrulanmadı</t>
-        </is>
-      </c>
-      <c r="H32" s="2" t="inlineStr">
-        <is>
-          <t>Google Workspace</t>
+          <t>üretildi – MX YOK, kesin bounce eder</t>
+        </is>
+      </c>
+      <c r="H32" s="3" t="inlineStr">
+        <is>
+          <t>MX YOK (MX kaydı yok)</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>HireFeed</t>
+          <t>Grid Studio</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>https://www.hirefeed.co.in</t>
+          <t>https://gridstudio.ai</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr"/>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>ik@hirefeed.co.in, kariyer@hirefeed.co.in, career@hirefeed.co.in, cv@hirefeed.co.in</t>
+          <t>ik@gridstudio.ai, kariyer@gridstudio.ai, career@gridstudio.ai, cv@gridstudio.ai</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>İK teknolojileri</t>
+          <t>Yapay zeka</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
@@ -1703,30 +1699,30 @@
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>var</t>
+          <t>Google Workspace</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>IAS - Canias ERP</t>
+          <t>Hepsiburada</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>https://www.caniaserp.com</t>
+          <t>https://www.hepsiburada.com</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr"/>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>ik@caniaserp.com, kariyer@caniaserp.com, career@caniaserp.com, cv@caniaserp.com</t>
+          <t>ik@hepsiburada.com, kariyer@hepsiburada.com, career@hepsiburada.com, cv@hepsiburada.com</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>ERP yazılımı</t>
+          <t>E-ticaret platformu</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
@@ -1741,35 +1737,35 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>var</t>
+          <t>Google Workspace</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>IdeaSoft</t>
+          <t>HireFeed</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>https://www.ideasoft.com.tr</t>
+          <t>https://www.hirefeed.co.in</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr"/>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>ik@ideasoft.com.tr, kariyer@ideasoft.com.tr, career@ideasoft.com.tr, cv@ideasoft.com.tr</t>
+          <t>ik@hirefeed.co.in, kariyer@hirefeed.co.in, career@hirefeed.co.in, cv@hirefeed.co.in</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>E-ticaret altyapı yazılımı</t>
+          <t>İK teknolojileri</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Kullanıcı listesi (05.08.2026)</t>
         </is>
       </c>
       <c r="G35" s="3" t="inlineStr">
@@ -1779,30 +1775,30 @@
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>Google Workspace</t>
+          <t>var</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>ininal</t>
+          <t>IAS - Canias ERP</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>https://www.ininal.com</t>
+          <t>https://www.caniaserp.com</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr"/>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>ik@ininal.com, kariyer@ininal.com, career@ininal.com, cv@ininal.com</t>
+          <t>ik@caniaserp.com, kariyer@caniaserp.com, career@caniaserp.com, cv@caniaserp.com</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Fintech / ön ödemeli kart</t>
+          <t>ERP yazılımı</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
@@ -1817,30 +1813,30 @@
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>Microsoft 365</t>
+          <t>var</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Innova Bilişim</t>
+          <t>IdeaSoft</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>https://www.innova.com.tr</t>
+          <t>https://www.ideasoft.com.tr</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr"/>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>ik@innova.com.tr, kariyer@innova.com.tr, career@innova.com.tr, cv@innova.com.tr</t>
+          <t>ik@ideasoft.com.tr, kariyer@ideasoft.com.tr, career@ideasoft.com.tr, cv@ideasoft.com.tr</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>BT çözümleri / sistem entegrasyonu</t>
+          <t>E-ticaret altyapı yazılımı</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
@@ -1855,30 +1851,30 @@
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>var</t>
+          <t>Google Workspace</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Insider</t>
+          <t>ininal</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>https://useinsider.com</t>
+          <t>https://www.ininal.com</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr"/>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>ik@useinsider.com, kariyer@useinsider.com, career@useinsider.com, cv@useinsider.com</t>
+          <t>ik@ininal.com, kariyer@ininal.com, career@ininal.com, cv@ininal.com</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Pazarlama teknolojileri / SaaS</t>
+          <t>Fintech / ön ödemeli kart</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
@@ -1893,30 +1889,30 @@
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>var</t>
+          <t>Microsoft 365</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Intertech</t>
+          <t>Innova Bilişim</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>https://www.intertech.com.tr</t>
+          <t>https://www.innova.com.tr</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr"/>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>ik@intertech.com.tr, kariyer@intertech.com.tr, career@intertech.com.tr, cv@intertech.com.tr</t>
+          <t>ik@innova.com.tr, kariyer@innova.com.tr, career@innova.com.tr, cv@innova.com.tr</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Bankacılık teknolojileri</t>
+          <t>BT çözümleri / sistem entegrasyonu</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
@@ -1938,23 +1934,23 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>iyzico</t>
+          <t>Insider</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>https://www.iyzico.com</t>
+          <t>https://useinsider.com</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr"/>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>ik@iyzico.com, kariyer@iyzico.com, career@iyzico.com, cv@iyzico.com</t>
+          <t>ik@useinsider.com, kariyer@useinsider.com, career@useinsider.com, cv@useinsider.com</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Fintech / ödeme sistemleri</t>
+          <t>Pazarlama teknolojileri / SaaS</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
@@ -1969,30 +1965,30 @@
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>Microsoft 365</t>
+          <t>var</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>İzibiz</t>
+          <t>Intertech</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>https://www.izibiz.com.tr</t>
+          <t>https://www.intertech.com.tr</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr"/>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>ik@izibiz.com.tr, kariyer@izibiz.com.tr, career@izibiz.com.tr, cv@izibiz.com.tr</t>
+          <t>ik@intertech.com.tr, kariyer@intertech.com.tr, career@intertech.com.tr, cv@intertech.com.tr</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>e-Fatura / e-dönüşüm</t>
+          <t>Bankacılık teknolojileri</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
@@ -2007,30 +2003,30 @@
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>Microsoft 365</t>
+          <t>var</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Kariyer.net</t>
+          <t>iyzico</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>https://www.kariyer.net</t>
+          <t>https://www.iyzico.com</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr"/>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>ik@kariyer.net, kariyer@kariyer.net, career@kariyer.net, cv@kariyer.net</t>
+          <t>ik@iyzico.com, kariyer@iyzico.com, career@iyzico.com, cv@iyzico.com</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>İK teknolojileri</t>
+          <t>Fintech / ödeme sistemleri</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
@@ -2052,23 +2048,23 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>KoçSistem</t>
+          <t>İzibiz</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>https://www.kocsistem.com.tr</t>
+          <t>https://www.izibiz.com.tr</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr"/>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>ik@kocsistem.com.tr, kariyer@kocsistem.com.tr, career@kocsistem.com.tr, cv@kocsistem.com.tr</t>
+          <t>ik@izibiz.com.tr, kariyer@izibiz.com.tr, career@izibiz.com.tr, cv@izibiz.com.tr</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>BT hizmetleri / sistem entegrasyonu</t>
+          <t>e-Fatura / e-dönüşüm</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
@@ -2083,30 +2079,30 @@
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>var</t>
+          <t>Microsoft 365</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Kron Technologies</t>
+          <t>Kariyer.net</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>https://krontech.com</t>
+          <t>https://www.kariyer.net</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr"/>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>ik@krontech.com, kariyer@krontech.com, career@krontech.com, cv@krontech.com</t>
+          <t>ik@kariyer.net, kariyer@kariyer.net, career@kariyer.net, cv@kariyer.net</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Siber güvenlik / erişim yönetimi</t>
+          <t>İK teknolojileri</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
@@ -2128,23 +2124,23 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>Link Bilgisayar</t>
+          <t>KoçSistem</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkbilgisayar.com.tr</t>
+          <t>https://www.kocsistem.com.tr</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr"/>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>ik@linkbilgisayar.com.tr, kariyer@linkbilgisayar.com.tr, career@linkbilgisayar.com.tr, cv@linkbilgisayar.com.tr</t>
+          <t>ik@kocsistem.com.tr, kariyer@kocsistem.com.tr, career@kocsistem.com.tr, cv@kocsistem.com.tr</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>Ticari yazılım</t>
+          <t>BT hizmetleri / sistem entegrasyonu</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
@@ -2159,35 +2155,35 @@
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>Microsoft 365</t>
+          <t>var</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Loodos</t>
+          <t>Kron Technologies</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>https://loodos.com</t>
+          <t>https://krontech.com</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr"/>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>ik@loodos.com, kariyer@loodos.com, career@loodos.com, cv@loodos.com</t>
+          <t>ik@krontech.com, kariyer@krontech.com, career@krontech.com, cv@krontech.com</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Mobil uygulama geliştirme</t>
+          <t>Siber güvenlik / erişim yönetimi</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>Kullanıcı listesi (05.08.2026)</t>
+          <t>Ön liste (doğrulanmadı)</t>
         </is>
       </c>
       <c r="G46" s="3" t="inlineStr">
@@ -2197,35 +2193,35 @@
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>Google Workspace</t>
+          <t>Microsoft 365</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>Lyrebird Studio</t>
+          <t>Link Bilgisayar</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>https://www.lyrebirdstudio.net</t>
+          <t>https://www.linkbilgisayar.com.tr</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr"/>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>ik@lyrebirdstudio.net, kariyer@lyrebirdstudio.net, career@lyrebirdstudio.net, cv@lyrebirdstudio.net</t>
+          <t>ik@linkbilgisayar.com.tr, kariyer@linkbilgisayar.com.tr, career@linkbilgisayar.com.tr, cv@linkbilgisayar.com.tr</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>Mobil uygulama / foto düzenleme</t>
+          <t>Ticari yazılım</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>Kullanıcı listesi (05.08.2026)</t>
+          <t>Ön liste (doğrulanmadı)</t>
         </is>
       </c>
       <c r="G47" s="3" t="inlineStr">
@@ -2235,35 +2231,35 @@
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>Google Workspace</t>
+          <t>Microsoft 365</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Martı</t>
+          <t>Loodos</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>https://www.marti.tech</t>
+          <t>https://loodos.com</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr"/>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>ik@marti.tech, kariyer@marti.tech, career@marti.tech, cv@marti.tech</t>
+          <t>ik@loodos.com, kariyer@loodos.com, career@loodos.com, cv@loodos.com</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>Mobilite teknolojileri</t>
+          <t>Mobil uygulama geliştirme</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Kullanıcı listesi (05.08.2026)</t>
         </is>
       </c>
       <c r="G48" s="3" t="inlineStr">
@@ -2273,35 +2269,35 @@
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>var</t>
+          <t>Google Workspace</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>Midas</t>
+          <t>Lyrebird Studio</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>https://www.getmidas.com</t>
+          <t>https://www.lyrebirdstudio.net</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr"/>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>ik@getmidas.com, kariyer@getmidas.com, career@getmidas.com, cv@getmidas.com</t>
+          <t>ik@lyrebirdstudio.net, kariyer@lyrebirdstudio.net, career@lyrebirdstudio.net, cv@lyrebirdstudio.net</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>Fintech / yatırım platformu</t>
+          <t>Mobil uygulama / foto düzenleme</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Kullanıcı listesi (05.08.2026)</t>
         </is>
       </c>
       <c r="G49" s="3" t="inlineStr">
@@ -2311,30 +2307,30 @@
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>var</t>
+          <t>Google Workspace</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Mikro Yazılım</t>
+          <t>Martı</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>https://www.mikro.com.tr</t>
+          <t>https://www.marti.tech</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr"/>
       <c r="D50" s="3" t="inlineStr">
         <is>
-          <t>ik@mikro.com.tr, kariyer@mikro.com.tr, career@mikro.com.tr, cv@mikro.com.tr</t>
+          <t>ik@marti.tech, kariyer@marti.tech, career@marti.tech, cv@marti.tech</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>Muhasebe / ERP yazılımı</t>
+          <t>Mobilite teknolojileri</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
@@ -2356,28 +2352,24 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>Mobiroller</t>
+          <t>Mee Apps</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>https://www.mobiroller.com</t>
+          <t>https://meeapps.com.tr</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr"/>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>ik@mobiroller.com, kariyer@mobiroller.com, career@mobiroller.com, cv@mobiroller.com</t>
-        </is>
-      </c>
-      <c r="E51" s="2" t="inlineStr">
-        <is>
-          <t>Mobil uygulama geliştirme platformu</t>
-        </is>
-      </c>
+          <t>ik@meeapps.com.tr, kariyer@meeapps.com.tr, career@meeapps.com.tr, cv@meeapps.com.tr</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr"/>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Kullanıcı listesi (05.08.2026 - 2. parti)</t>
         </is>
       </c>
       <c r="G51" s="3" t="inlineStr">
@@ -2394,23 +2386,23 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>Mobven</t>
+          <t>Midas</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>https://mobven.com</t>
+          <t>https://www.getmidas.com</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr"/>
       <c r="D52" s="3" t="inlineStr">
         <is>
-          <t>ik@mobven.com, kariyer@mobven.com, career@mobven.com, cv@mobven.com</t>
+          <t>ik@getmidas.com, kariyer@getmidas.com, career@getmidas.com, cv@getmidas.com</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>Mobil yazılım geliştirme</t>
+          <t>Fintech / yatırım platformu</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
@@ -2425,30 +2417,30 @@
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>Google Workspace</t>
+          <t>var</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>Modanisa</t>
+          <t>Mikro Yazılım</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>https://www.modanisa.com</t>
+          <t>https://www.mikro.com.tr</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr"/>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>ik@modanisa.com, kariyer@modanisa.com, career@modanisa.com, cv@modanisa.com</t>
+          <t>ik@mikro.com.tr, kariyer@mikro.com.tr, career@mikro.com.tr, cv@mikro.com.tr</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>E-ticaret</t>
+          <t>Muhasebe / ERP yazılımı</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
@@ -2463,35 +2455,35 @@
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
-          <t>Google Workspace</t>
+          <t>var</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>Mono Dijital</t>
+          <t>Mobiroller</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>https://monodijital.com</t>
+          <t>https://www.mobiroller.com</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr"/>
       <c r="D54" s="3" t="inlineStr">
         <is>
-          <t>ik@monodijital.com, kariyer@monodijital.com, career@monodijital.com, cv@monodijital.com</t>
+          <t>ik@mobiroller.com, kariyer@mobiroller.com, career@mobiroller.com, cv@mobiroller.com</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>Dijital ajans</t>
+          <t>Mobil uygulama geliştirme platformu</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>Kullanıcı listesi (05.08.2026)</t>
+          <t>Ön liste (doğrulanmadı)</t>
         </is>
       </c>
       <c r="G54" s="3" t="inlineStr">
@@ -2501,35 +2493,35 @@
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>Yandex</t>
+          <t>Google Workspace</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>Native Minds</t>
+          <t>Mobven</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>https://nativeminds.ai</t>
+          <t>https://mobven.com</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr"/>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t>ik@nativeminds.ai, kariyer@nativeminds.ai, career@nativeminds.ai, cv@nativeminds.ai</t>
+          <t>ik@mobven.com, kariyer@mobven.com, career@mobven.com, cv@mobven.com</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>Yapay zeka</t>
+          <t>Mobil yazılım geliştirme</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>Kullanıcı listesi (05.08.2026)</t>
+          <t>Ön liste (doğrulanmadı)</t>
         </is>
       </c>
       <c r="G55" s="3" t="inlineStr">
@@ -2546,23 +2538,23 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>Nebim</t>
+          <t>Modanisa</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>https://www.nebim.com.tr</t>
+          <t>https://www.modanisa.com</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr"/>
       <c r="D56" s="3" t="inlineStr">
         <is>
-          <t>ik@nebim.com.tr, kariyer@nebim.com.tr, career@nebim.com.tr, cv@nebim.com.tr</t>
+          <t>ik@modanisa.com, kariyer@modanisa.com, career@modanisa.com, cv@modanisa.com</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>Perakende ERP yazılımı</t>
+          <t>E-ticaret</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
@@ -2584,23 +2576,23 @@
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>Neon Apps</t>
+          <t>Mono Dijital</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>https://neonapps.co</t>
+          <t>https://monodijital.com</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr"/>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t>ik@neonapps.co, kariyer@neonapps.co, career@neonapps.co, cv@neonapps.co</t>
+          <t>ik@monodijital.com, kariyer@monodijital.com, career@monodijital.com, cv@monodijital.com</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>Mobil uygulama geliştirme</t>
+          <t>Dijital ajans</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
@@ -2615,35 +2607,35 @@
       </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
-          <t>Google Workspace</t>
+          <t>Yandex</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>Netaş</t>
+          <t>Native Minds</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>https://www.netas.com.tr</t>
+          <t>https://nativeminds.ai</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr"/>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t>ik@netas.com.tr, kariyer@netas.com.tr, career@netas.com.tr, cv@netas.com.tr</t>
+          <t>ik@nativeminds.ai, kariyer@nativeminds.ai, career@nativeminds.ai, cv@nativeminds.ai</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>Telekom ve yazılım çözümleri</t>
+          <t>Yapay zeka</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Kullanıcı listesi (05.08.2026)</t>
         </is>
       </c>
       <c r="G58" s="3" t="inlineStr">
@@ -2653,35 +2645,35 @@
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>Microsoft 365</t>
+          <t>Google Workspace</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>NGaming</t>
+          <t>Nebim</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>https://ngaming.com</t>
+          <t>https://www.nebim.com.tr</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr"/>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>ik@ngaming.com, kariyer@ngaming.com, career@ngaming.com, cv@ngaming.com</t>
+          <t>ik@nebim.com.tr, kariyer@nebim.com.tr, career@nebim.com.tr, cv@nebim.com.tr</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>Oyun</t>
+          <t>Perakende ERP yazılımı</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>Kullanıcı listesi (05.08.2026)</t>
+          <t>Ön liste (doğrulanmadı)</t>
         </is>
       </c>
       <c r="G59" s="3" t="inlineStr">
@@ -2691,28 +2683,32 @@
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t>Microsoft 365</t>
+          <t>Google Workspace</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>Oak Technology</t>
+          <t>Neon Apps</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>https://oak.technology</t>
+          <t>https://neonapps.co</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr"/>
       <c r="D60" s="3" t="inlineStr">
         <is>
-          <t>ik@oak.technology, kariyer@oak.technology, career@oak.technology, cv@oak.technology</t>
-        </is>
-      </c>
-      <c r="E60" s="2" t="inlineStr"/>
+          <t>ik@neonapps.co, kariyer@neonapps.co, career@neonapps.co, cv@neonapps.co</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>Mobil uygulama geliştirme</t>
+        </is>
+      </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
           <t>Kullanıcı listesi (05.08.2026)</t>
@@ -2725,35 +2721,31 @@
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>var</t>
+          <t>Google Workspace</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>OBSS</t>
+          <t>Neova</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>https://obss.tech</t>
+          <t>https://neova.com.tr</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr"/>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t>ik@obss.tech, kariyer@obss.tech, career@obss.tech, cv@obss.tech</t>
-        </is>
-      </c>
-      <c r="E61" s="2" t="inlineStr">
-        <is>
-          <t>Yazılım geliştirme / danışmanlık</t>
-        </is>
-      </c>
+          <t>ik@neova.com.tr, kariyer@neova.com.tr, career@neova.com.tr, cv@neova.com.tr</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr"/>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Kullanıcı listesi (05.08.2026 - 2. parti)</t>
         </is>
       </c>
       <c r="G61" s="3" t="inlineStr">
@@ -2763,30 +2755,30 @@
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
-          <t>Google Workspace</t>
+          <t>var</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>Papara</t>
+          <t>Netaş</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>https://www.papara.com</t>
+          <t>https://www.netas.com.tr</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr"/>
       <c r="D62" s="3" t="inlineStr">
         <is>
-          <t>ik@papara.com, kariyer@papara.com, career@papara.com, cv@papara.com</t>
+          <t>ik@netas.com.tr, kariyer@netas.com.tr, career@netas.com.tr, cv@netas.com.tr</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>Fintech / dijital cüzdan</t>
+          <t>Telekom ve yazılım çözümleri</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
@@ -2808,28 +2800,28 @@
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>Param</t>
+          <t>NGaming</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>https://www.param.com.tr</t>
+          <t>https://ngaming.com</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr"/>
       <c r="D63" s="3" t="inlineStr">
         <is>
-          <t>ik@param.com.tr, kariyer@param.com.tr, career@param.com.tr, cv@param.com.tr</t>
+          <t>ik@ngaming.com, kariyer@ngaming.com, career@ngaming.com, cv@ngaming.com</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>Fintech / ödeme sistemleri</t>
+          <t>Oyun</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Kullanıcı listesi (05.08.2026)</t>
         </is>
       </c>
       <c r="G63" s="3" t="inlineStr">
@@ -2839,35 +2831,31 @@
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
-          <t>Google Workspace</t>
+          <t>Microsoft 365</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>Paribu</t>
+          <t>Oak Technology</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>https://www.paribu.com</t>
+          <t>https://oak.technology</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr"/>
       <c r="D64" s="3" t="inlineStr">
         <is>
-          <t>ik@paribu.com, kariyer@paribu.com, career@paribu.com, cv@paribu.com</t>
-        </is>
-      </c>
-      <c r="E64" s="2" t="inlineStr">
-        <is>
-          <t>Kripto varlık platformu</t>
-        </is>
-      </c>
+          <t>ik@oak.technology, kariyer@oak.technology, career@oak.technology, cv@oak.technology</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr"/>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Kullanıcı listesi (05.08.2026)</t>
         </is>
       </c>
       <c r="G64" s="3" t="inlineStr">
@@ -2877,30 +2865,30 @@
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t>Google Workspace</t>
+          <t>var</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>PayCore</t>
+          <t>OBSS</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>https://www.paycore.com</t>
+          <t>https://obss.tech</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr"/>
       <c r="D65" s="3" t="inlineStr">
         <is>
-          <t>ik@paycore.com, kariyer@paycore.com, career@paycore.com, cv@paycore.com</t>
+          <t>ik@obss.tech, kariyer@obss.tech, career@obss.tech, cv@obss.tech</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>Fintech / kart teknolojileri</t>
+          <t>Yazılım geliştirme / danışmanlık</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
@@ -2915,30 +2903,30 @@
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
-          <t>Microsoft 365</t>
+          <t>Google Workspace</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>Peak Games</t>
+          <t>Papara</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>https://www.peak.com</t>
+          <t>https://www.papara.com</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr"/>
       <c r="D66" s="3" t="inlineStr">
         <is>
-          <t>ik@peak.com, kariyer@peak.com, career@peak.com, cv@peak.com</t>
+          <t>ik@papara.com, kariyer@papara.com, career@papara.com, cv@papara.com</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>Mobil oyun</t>
+          <t>Fintech / dijital cüzdan</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
@@ -2953,30 +2941,30 @@
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
-          <t>Google Workspace</t>
+          <t>Microsoft 365</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>Platin Bilişim</t>
+          <t>Param</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>https://www.platinbilisim.com.tr</t>
+          <t>https://www.param.com.tr</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr"/>
       <c r="D67" s="3" t="inlineStr">
         <is>
-          <t>ik@platinbilisim.com.tr, kariyer@platinbilisim.com.tr, career@platinbilisim.com.tr, cv@platinbilisim.com.tr</t>
+          <t>ik@param.com.tr, kariyer@param.com.tr, career@param.com.tr, cv@param.com.tr</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>BT çözümleri / sistem entegrasyonu</t>
+          <t>Fintech / ödeme sistemleri</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
@@ -2991,35 +2979,35 @@
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
-          <t>Microsoft 365</t>
+          <t>Google Workspace</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>Playable Factory</t>
+          <t>Paribu</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>https://playablefactory.com</t>
+          <t>https://www.paribu.com</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr"/>
       <c r="D68" s="3" t="inlineStr">
         <is>
-          <t>ik@playablefactory.com, kariyer@playablefactory.com, career@playablefactory.com, cv@playablefactory.com</t>
+          <t>ik@paribu.com, kariyer@paribu.com, career@paribu.com, cv@paribu.com</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>Oynanabilir reklam / oyun teknolojisi</t>
+          <t>Kripto varlık platformu</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>Kullanıcı listesi (05.08.2026)</t>
+          <t>Ön liste (doğrulanmadı)</t>
         </is>
       </c>
       <c r="G68" s="3" t="inlineStr">
@@ -3036,23 +3024,23 @@
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>Protel</t>
+          <t>PayCore</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>https://www.protel.com.tr</t>
+          <t>https://www.paycore.com</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr"/>
       <c r="D69" s="3" t="inlineStr">
         <is>
-          <t>ik@protel.com.tr, kariyer@protel.com.tr, career@protel.com.tr, cv@protel.com.tr</t>
+          <t>ik@paycore.com, kariyer@paycore.com, career@paycore.com, cv@paycore.com</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>Otel ve restoran yazılımı</t>
+          <t>Fintech / kart teknolojileri</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
@@ -3067,35 +3055,31 @@
       </c>
       <c r="H69" s="2" t="inlineStr">
         <is>
-          <t>Google Workspace</t>
+          <t>Microsoft 365</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>Related Digital</t>
+          <t>Paymore</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>https://www.relateddigital.com</t>
+          <t>https://paymore.com.tr</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr"/>
       <c r="D70" s="3" t="inlineStr">
         <is>
-          <t>ik@relateddigital.com, kariyer@relateddigital.com, career@relateddigital.com, cv@relateddigital.com</t>
-        </is>
-      </c>
-      <c r="E70" s="2" t="inlineStr">
-        <is>
-          <t>Pazarlama teknolojileri</t>
-        </is>
-      </c>
+          <t>ik@paymore.com.tr, kariyer@paymore.com.tr, career@paymore.com.tr, cv@paymore.com.tr</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="inlineStr"/>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Kullanıcı listesi (05.08.2026 - 2. parti)</t>
         </is>
       </c>
       <c r="G70" s="3" t="inlineStr">
@@ -3105,35 +3089,35 @@
       </c>
       <c r="H70" s="2" t="inlineStr">
         <is>
-          <t>Microsoft 365</t>
+          <t>Google Workspace</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>Rentcarla</t>
+          <t>Peak Games</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>https://rentcarla.com</t>
+          <t>https://www.peak.com</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr"/>
       <c r="D71" s="3" t="inlineStr">
         <is>
-          <t>ik@rentcarla.com, kariyer@rentcarla.com, career@rentcarla.com, cv@rentcarla.com</t>
+          <t>ik@peak.com, kariyer@peak.com, career@peak.com, cv@peak.com</t>
         </is>
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>Araç kiralama platformu</t>
+          <t>Mobil oyun</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>Kullanıcı listesi (05.08.2026)</t>
+          <t>Ön liste (doğrulanmadı)</t>
         </is>
       </c>
       <c r="G71" s="3" t="inlineStr">
@@ -3150,23 +3134,23 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>Rollic Games</t>
+          <t>Platin Bilişim</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>https://www.rollicgames.com</t>
+          <t>https://www.platinbilisim.com.tr</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr"/>
       <c r="D72" s="3" t="inlineStr">
         <is>
-          <t>ik@rollicgames.com, kariyer@rollicgames.com, career@rollicgames.com, cv@rollicgames.com</t>
+          <t>ik@platinbilisim.com.tr, kariyer@platinbilisim.com.tr, career@platinbilisim.com.tr, cv@platinbilisim.com.tr</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>Mobil oyun</t>
+          <t>BT çözümleri / sistem entegrasyonu</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
@@ -3181,35 +3165,35 @@
       </c>
       <c r="H72" s="2" t="inlineStr">
         <is>
-          <t>Google Workspace</t>
+          <t>Microsoft 365</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>Sabancı DX</t>
+          <t>Playable Factory</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>https://www.sabancidx.com</t>
+          <t>https://playablefactory.com</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr"/>
       <c r="D73" s="3" t="inlineStr">
         <is>
-          <t>ik@sabancidx.com, kariyer@sabancidx.com, career@sabancidx.com, cv@sabancidx.com</t>
+          <t>ik@playablefactory.com, kariyer@playablefactory.com, career@playablefactory.com, cv@playablefactory.com</t>
         </is>
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>Dijital teknoloji / veri</t>
+          <t>Oynanabilir reklam / oyun teknolojisi</t>
         </is>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Kullanıcı listesi (05.08.2026)</t>
         </is>
       </c>
       <c r="G73" s="3" t="inlineStr">
@@ -3219,30 +3203,30 @@
       </c>
       <c r="H73" s="2" t="inlineStr">
         <is>
-          <t>var</t>
+          <t>Google Workspace</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>Sahibinden.com</t>
+          <t>Protel</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>https://www.sahibinden.com</t>
+          <t>https://www.protel.com.tr</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr"/>
       <c r="D74" s="3" t="inlineStr">
         <is>
-          <t>ik@sahibinden.com, kariyer@sahibinden.com, career@sahibinden.com, cv@sahibinden.com</t>
+          <t>ik@protel.com.tr, kariyer@protel.com.tr, career@protel.com.tr, cv@protel.com.tr</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>Online ilan platformu</t>
+          <t>Otel ve restoran yazılımı</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
@@ -3257,30 +3241,30 @@
       </c>
       <c r="H74" s="2" t="inlineStr">
         <is>
-          <t>Microsoft 365</t>
+          <t>Google Workspace</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>Segmentify</t>
+          <t>Related Digital</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>https://www.segmentify.com</t>
+          <t>https://www.relateddigital.com</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr"/>
       <c r="D75" s="3" t="inlineStr">
         <is>
-          <t>ik@segmentify.com, kariyer@segmentify.com, career@segmentify.com, cv@segmentify.com</t>
+          <t>ik@relateddigital.com, kariyer@relateddigital.com, career@relateddigital.com, cv@relateddigital.com</t>
         </is>
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>E-ticaret kişiselleştirme</t>
+          <t>Pazarlama teknolojileri</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
@@ -3295,35 +3279,35 @@
       </c>
       <c r="H75" s="2" t="inlineStr">
         <is>
-          <t>Google Workspace</t>
+          <t>Microsoft 365</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>Setrow</t>
+          <t>Rentcarla</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>https://setrow.com</t>
+          <t>https://rentcarla.com</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr"/>
       <c r="D76" s="3" t="inlineStr">
         <is>
-          <t>ik@setrow.com, kariyer@setrow.com, career@setrow.com, cv@setrow.com</t>
+          <t>ik@rentcarla.com, kariyer@rentcarla.com, career@rentcarla.com, cv@rentcarla.com</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>E-posta pazarlama teknolojisi</t>
+          <t>Araç kiralama platformu</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Kullanıcı listesi (05.08.2026)</t>
         </is>
       </c>
       <c r="G76" s="3" t="inlineStr">
@@ -3333,35 +3317,35 @@
       </c>
       <c r="H76" s="2" t="inlineStr">
         <is>
-          <t>Microsoft 365</t>
+          <t>Google Workspace</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>Seven Apps</t>
+          <t>Rollic Games</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>https://sevenapps.co</t>
+          <t>https://www.rollicgames.com</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr"/>
       <c r="D77" s="3" t="inlineStr">
         <is>
-          <t>ik@sevenapps.co, kariyer@sevenapps.co, career@sevenapps.co, cv@sevenapps.co</t>
+          <t>ik@rollicgames.com, kariyer@rollicgames.com, career@rollicgames.com, cv@rollicgames.com</t>
         </is>
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>Mobil uygulama geliştirme</t>
+          <t>Mobil oyun</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>Kullanıcı listesi (05.08.2026)</t>
+          <t>Ön liste (doğrulanmadı)</t>
         </is>
       </c>
       <c r="G77" s="3" t="inlineStr">
@@ -3378,23 +3362,23 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>Sipay</t>
+          <t>Sabancı DX</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>https://www.sipay.com.tr</t>
+          <t>https://www.sabancidx.com</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr"/>
       <c r="D78" s="3" t="inlineStr">
         <is>
-          <t>ik@sipay.com.tr, kariyer@sipay.com.tr, career@sipay.com.tr, cv@sipay.com.tr</t>
+          <t>ik@sabancidx.com, kariyer@sabancidx.com, career@sabancidx.com, cv@sabancidx.com</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>Fintech / ödeme sistemleri</t>
+          <t>Dijital teknoloji / veri</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
@@ -3409,30 +3393,30 @@
       </c>
       <c r="H78" s="2" t="inlineStr">
         <is>
-          <t>Microsoft 365</t>
+          <t>var</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>Sistaş</t>
+          <t>Sahibinden.com</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>https://www.sistas.com.tr</t>
+          <t>https://www.sahibinden.com</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr"/>
       <c r="D79" s="3" t="inlineStr">
         <is>
-          <t>ik@sistas.com.tr, kariyer@sistas.com.tr, career@sistas.com.tr, cv@sistas.com.tr</t>
+          <t>ik@sahibinden.com, kariyer@sahibinden.com, career@sahibinden.com, cv@sahibinden.com</t>
         </is>
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>BT çözümleri</t>
+          <t>Online ilan platformu</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr">
@@ -3447,35 +3431,35 @@
       </c>
       <c r="H79" s="2" t="inlineStr">
         <is>
-          <t>var</t>
+          <t>Microsoft 365</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>Slayz</t>
+          <t>Segmentify</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>https://slayz.app</t>
+          <t>https://www.segmentify.com</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr"/>
       <c r="D80" s="3" t="inlineStr">
         <is>
-          <t>ik@slayz.app, kariyer@slayz.app, career@slayz.app, cv@slayz.app</t>
+          <t>ik@segmentify.com, kariyer@segmentify.com, career@segmentify.com, cv@segmentify.com</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>Mobil uygulama</t>
+          <t>E-ticaret kişiselleştirme</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>Kullanıcı listesi (05.08.2026)</t>
+          <t>Ön liste (doğrulanmadı)</t>
         </is>
       </c>
       <c r="G80" s="3" t="inlineStr">
@@ -3485,35 +3469,31 @@
       </c>
       <c r="H80" s="2" t="inlineStr">
         <is>
-          <t>Microsoft 365</t>
+          <t>Google Workspace</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>Softtech</t>
+          <t>ServiceCore</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>https://www.softtech.com.tr</t>
+          <t>https://servicecore.app</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr"/>
       <c r="D81" s="3" t="inlineStr">
         <is>
-          <t>ik@softtech.com.tr, kariyer@softtech.com.tr, career@softtech.com.tr, cv@softtech.com.tr</t>
-        </is>
-      </c>
-      <c r="E81" s="2" t="inlineStr">
-        <is>
-          <t>Bankacılık yazılımı</t>
-        </is>
-      </c>
+          <t>ik@servicecore.app, kariyer@servicecore.app, career@servicecore.app, cv@servicecore.app</t>
+        </is>
+      </c>
+      <c r="E81" s="2" t="inlineStr"/>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Kullanıcı listesi (05.08.2026 - 2. parti)</t>
         </is>
       </c>
       <c r="G81" s="3" t="inlineStr">
@@ -3530,23 +3510,23 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>Spyke Games</t>
+          <t>Setrow</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>https://www.spykegames.com</t>
+          <t>https://setrow.com</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr"/>
       <c r="D82" s="3" t="inlineStr">
         <is>
-          <t>ik@spykegames.com, kariyer@spykegames.com, career@spykegames.com, cv@spykegames.com</t>
+          <t>ik@setrow.com, kariyer@setrow.com, career@setrow.com, cv@setrow.com</t>
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>Mobil oyun</t>
+          <t>E-posta pazarlama teknolojisi</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
@@ -3561,35 +3541,35 @@
       </c>
       <c r="H82" s="2" t="inlineStr">
         <is>
-          <t>Google Workspace</t>
+          <t>Microsoft 365</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>T-Soft</t>
+          <t>Seven Apps</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>https://www.tsoft.com.tr</t>
+          <t>https://sevenapps.co</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr"/>
       <c r="D83" s="3" t="inlineStr">
         <is>
-          <t>ik@tsoft.com.tr, kariyer@tsoft.com.tr, career@tsoft.com.tr, cv@tsoft.com.tr</t>
+          <t>ik@sevenapps.co, kariyer@sevenapps.co, career@sevenapps.co, cv@sevenapps.co</t>
         </is>
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>E-ticaret yazılımı</t>
+          <t>Mobil uygulama geliştirme</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Kullanıcı listesi (05.08.2026)</t>
         </is>
       </c>
       <c r="G83" s="3" t="inlineStr">
@@ -3599,31 +3579,35 @@
       </c>
       <c r="H83" s="2" t="inlineStr">
         <is>
-          <t>var</t>
+          <t>Google Workspace</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>TankX</t>
+          <t>Shipday</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>https://tankx.co</t>
+          <t>https://shipday.com</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr"/>
       <c r="D84" s="3" t="inlineStr">
         <is>
-          <t>ik@tankx.co, kariyer@tankx.co, career@tankx.co, cv@tankx.co</t>
-        </is>
-      </c>
-      <c r="E84" s="2" t="inlineStr"/>
+          <t>ik@shipday.com, kariyer@shipday.com, career@shipday.com, cv@shipday.com</t>
+        </is>
+      </c>
+      <c r="E84" s="2" t="inlineStr">
+        <is>
+          <t>Teslimat yönetimi yazılımı</t>
+        </is>
+      </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>Kullanıcı listesi (05.08.2026)</t>
+          <t>Kullanıcı listesi (05.08.2026 - 2. parti)</t>
         </is>
       </c>
       <c r="G84" s="3" t="inlineStr">
@@ -3640,23 +3624,23 @@
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>Testinium</t>
+          <t>Sipay</t>
         </is>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>https://testinium.com</t>
+          <t>https://www.sipay.com.tr</t>
         </is>
       </c>
       <c r="C85" s="2" t="inlineStr"/>
       <c r="D85" s="3" t="inlineStr">
         <is>
-          <t>ik@testinium.com, kariyer@testinium.com, career@testinium.com, cv@testinium.com</t>
+          <t>ik@sipay.com.tr, kariyer@sipay.com.tr, career@sipay.com.tr, cv@sipay.com.tr</t>
         </is>
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>Test otomasyonu / yazılım kalite</t>
+          <t>Fintech / ödeme sistemleri</t>
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr">
@@ -3678,23 +3662,23 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>Ticimax</t>
+          <t>Sistaş</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>https://www.ticimax.com</t>
+          <t>https://www.sistas.com.tr</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr"/>
       <c r="D86" s="3" t="inlineStr">
         <is>
-          <t>ik@ticimax.com, kariyer@ticimax.com, career@ticimax.com, cv@ticimax.com</t>
+          <t>ik@sistas.com.tr, kariyer@sistas.com.tr, career@sistas.com.tr, cv@sistas.com.tr</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>E-ticaret altyapı yazılımı</t>
+          <t>BT çözümleri</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">
@@ -3709,35 +3693,35 @@
       </c>
       <c r="H86" s="2" t="inlineStr">
         <is>
-          <t>Microsoft 365</t>
+          <t>var</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>Trendyol</t>
+          <t>Slayz</t>
         </is>
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>https://www.trendyol.com</t>
+          <t>https://slayz.app</t>
         </is>
       </c>
       <c r="C87" s="2" t="inlineStr"/>
       <c r="D87" s="3" t="inlineStr">
         <is>
-          <t>ik@trendyol.com, kariyer@trendyol.com, career@trendyol.com, cv@trendyol.com</t>
+          <t>ik@slayz.app, kariyer@slayz.app, career@slayz.app, cv@slayz.app</t>
         </is>
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>E-ticaret platformu</t>
+          <t>Mobil uygulama</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Kullanıcı listesi (05.08.2026)</t>
         </is>
       </c>
       <c r="G87" s="3" t="inlineStr">
@@ -3747,30 +3731,30 @@
       </c>
       <c r="H87" s="2" t="inlineStr">
         <is>
-          <t>var</t>
+          <t>Microsoft 365</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>Uyumsoft</t>
+          <t>Softtech</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>https://www.uyumsoft.com.tr</t>
+          <t>https://www.softtech.com.tr</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr"/>
       <c r="D88" s="3" t="inlineStr">
         <is>
-          <t>ik@uyumsoft.com.tr, kariyer@uyumsoft.com.tr, career@uyumsoft.com.tr, cv@uyumsoft.com.tr</t>
+          <t>ik@softtech.com.tr, kariyer@softtech.com.tr, career@softtech.com.tr, cv@softtech.com.tr</t>
         </is>
       </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
-          <t>ERP / e-dönüşüm yazılımı</t>
+          <t>Bankacılık yazılımı</t>
         </is>
       </c>
       <c r="F88" s="2" t="inlineStr">
@@ -3785,35 +3769,35 @@
       </c>
       <c r="H88" s="2" t="inlineStr">
         <is>
-          <t>Microsoft 365</t>
+          <t>var</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>VeriPark</t>
+          <t>Solvoyo</t>
         </is>
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>https://www.veripark.com</t>
+          <t>https://solvoyo.com</t>
         </is>
       </c>
       <c r="C89" s="2" t="inlineStr"/>
       <c r="D89" s="3" t="inlineStr">
         <is>
-          <t>ik@veripark.com, kariyer@veripark.com, career@veripark.com, cv@veripark.com</t>
+          <t>ik@solvoyo.com, kariyer@solvoyo.com, career@solvoyo.com, cv@solvoyo.com</t>
         </is>
       </c>
       <c r="E89" s="2" t="inlineStr">
         <is>
-          <t>Bankacılık yazılımı</t>
+          <t>Tedarik zinciri planlama / yapay zeka</t>
         </is>
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Kullanıcı listesi (05.08.2026 - 2. parti)</t>
         </is>
       </c>
       <c r="G89" s="3" t="inlineStr">
@@ -3823,35 +3807,35 @@
       </c>
       <c r="H89" s="2" t="inlineStr">
         <is>
-          <t>Microsoft 365</t>
+          <t>Google Workspace</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>Virgosol</t>
+          <t>Spyke Games</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>https://virgosol.com</t>
+          <t>https://www.spykegames.com</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr"/>
       <c r="D90" s="3" t="inlineStr">
         <is>
-          <t>ik@virgosol.com, kariyer@virgosol.com, career@virgosol.com, cv@virgosol.com</t>
+          <t>ik@spykegames.com, kariyer@spykegames.com, career@spykegames.com, cv@spykegames.com</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
         <is>
-          <t>Yazılım geliştirme</t>
+          <t>Mobil oyun</t>
         </is>
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
-          <t>Kullanıcı listesi (05.08.2026)</t>
+          <t>Ön liste (doğrulanmadı)</t>
         </is>
       </c>
       <c r="G90" s="3" t="inlineStr">
@@ -3861,30 +3845,30 @@
       </c>
       <c r="H90" s="2" t="inlineStr">
         <is>
-          <t>Microsoft 365</t>
+          <t>Google Workspace</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>Vispera</t>
+          <t>T-Soft</t>
         </is>
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>https://vispera.co</t>
+          <t>https://www.tsoft.com.tr</t>
         </is>
       </c>
       <c r="C91" s="2" t="inlineStr"/>
       <c r="D91" s="3" t="inlineStr">
         <is>
-          <t>ik@vispera.co, kariyer@vispera.co, career@vispera.co, cv@vispera.co</t>
+          <t>ik@tsoft.com.tr, kariyer@tsoft.com.tr, career@tsoft.com.tr, cv@tsoft.com.tr</t>
         </is>
       </c>
       <c r="E91" s="2" t="inlineStr">
         <is>
-          <t>Yapay zeka / görüntü işleme</t>
+          <t>E-ticaret yazılımı</t>
         </is>
       </c>
       <c r="F91" s="2" t="inlineStr">
@@ -3899,32 +3883,28 @@
       </c>
       <c r="H91" s="2" t="inlineStr">
         <is>
-          <t>Microsoft 365</t>
+          <t>var</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>VoltLines</t>
+          <t>TankX</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>https://voltlines.com</t>
+          <t>https://tankx.co</t>
         </is>
       </c>
       <c r="C92" s="2" t="inlineStr"/>
       <c r="D92" s="3" t="inlineStr">
         <is>
-          <t>ik@voltlines.com, kariyer@voltlines.com, career@voltlines.com, cv@voltlines.com</t>
-        </is>
-      </c>
-      <c r="E92" s="2" t="inlineStr">
-        <is>
-          <t>Kurumsal ulaşım teknolojisi</t>
-        </is>
-      </c>
+          <t>ik@tankx.co, kariyer@tankx.co, career@tankx.co, cv@tankx.co</t>
+        </is>
+      </c>
+      <c r="E92" s="2" t="inlineStr"/>
       <c r="F92" s="2" t="inlineStr">
         <is>
           <t>Kullanıcı listesi (05.08.2026)</t>
@@ -3944,23 +3924,23 @@
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>Workcube</t>
+          <t>Testinium</t>
         </is>
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>https://www.workcube.com</t>
+          <t>https://testinium.com</t>
         </is>
       </c>
       <c r="C93" s="2" t="inlineStr"/>
       <c r="D93" s="3" t="inlineStr">
         <is>
-          <t>ik@workcube.com, kariyer@workcube.com, career@workcube.com, cv@workcube.com</t>
+          <t>ik@testinium.com, kariyer@testinium.com, career@testinium.com, cv@testinium.com</t>
         </is>
       </c>
       <c r="E93" s="2" t="inlineStr">
         <is>
-          <t>Kurumsal yazılım / ERP</t>
+          <t>Test otomasyonu / yazılım kalite</t>
         </is>
       </c>
       <c r="F93" s="2" t="inlineStr">
@@ -3975,50 +3955,426 @@
       </c>
       <c r="H93" s="2" t="inlineStr">
         <is>
-          <t>Google Workspace</t>
+          <t>Microsoft 365</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>Yemeksepeti</t>
+          <t>Ticimax</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>https://www.yemeksepeti.com</t>
+          <t>https://www.ticimax.com</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr"/>
       <c r="D94" s="3" t="inlineStr">
         <is>
+          <t>ik@ticimax.com, kariyer@ticimax.com, career@ticimax.com, cv@ticimax.com</t>
+        </is>
+      </c>
+      <c r="E94" s="2" t="inlineStr">
+        <is>
+          <t>E-ticaret altyapı yazılımı</t>
+        </is>
+      </c>
+      <c r="F94" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G94" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
+        </is>
+      </c>
+      <c r="H94" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft 365</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="inlineStr">
+        <is>
+          <t>Trendyol</t>
+        </is>
+      </c>
+      <c r="B95" s="2" t="inlineStr">
+        <is>
+          <t>https://www.trendyol.com</t>
+        </is>
+      </c>
+      <c r="C95" s="2" t="inlineStr"/>
+      <c r="D95" s="3" t="inlineStr">
+        <is>
+          <t>ik@trendyol.com, kariyer@trendyol.com, career@trendyol.com, cv@trendyol.com</t>
+        </is>
+      </c>
+      <c r="E95" s="2" t="inlineStr">
+        <is>
+          <t>E-ticaret platformu</t>
+        </is>
+      </c>
+      <c r="F95" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G95" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
+        </is>
+      </c>
+      <c r="H95" s="2" t="inlineStr">
+        <is>
+          <t>var</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="inlineStr">
+        <is>
+          <t>Uyumsoft</t>
+        </is>
+      </c>
+      <c r="B96" s="2" t="inlineStr">
+        <is>
+          <t>https://www.uyumsoft.com.tr</t>
+        </is>
+      </c>
+      <c r="C96" s="2" t="inlineStr"/>
+      <c r="D96" s="3" t="inlineStr">
+        <is>
+          <t>ik@uyumsoft.com.tr, kariyer@uyumsoft.com.tr, career@uyumsoft.com.tr, cv@uyumsoft.com.tr</t>
+        </is>
+      </c>
+      <c r="E96" s="2" t="inlineStr">
+        <is>
+          <t>ERP / e-dönüşüm yazılımı</t>
+        </is>
+      </c>
+      <c r="F96" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G96" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
+        </is>
+      </c>
+      <c r="H96" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft 365</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="inlineStr">
+        <is>
+          <t>Uyumsoft (.com)</t>
+        </is>
+      </c>
+      <c r="B97" s="2" t="inlineStr">
+        <is>
+          <t>https://uyumsoft.com</t>
+        </is>
+      </c>
+      <c r="C97" s="2" t="inlineStr"/>
+      <c r="D97" s="3" t="inlineStr">
+        <is>
+          <t>ik@uyumsoft.com, kariyer@uyumsoft.com, career@uyumsoft.com, cv@uyumsoft.com</t>
+        </is>
+      </c>
+      <c r="E97" s="2" t="inlineStr">
+        <is>
+          <t>ERP / e-dönüşüm yazılımı</t>
+        </is>
+      </c>
+      <c r="F97" s="2" t="inlineStr">
+        <is>
+          <t>Kullanıcı listesi (05.08.2026 - 2. parti)</t>
+        </is>
+      </c>
+      <c r="G97" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
+        </is>
+      </c>
+      <c r="H97" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft 365</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t>VeriPark</t>
+        </is>
+      </c>
+      <c r="B98" s="2" t="inlineStr">
+        <is>
+          <t>https://www.veripark.com</t>
+        </is>
+      </c>
+      <c r="C98" s="2" t="inlineStr"/>
+      <c r="D98" s="3" t="inlineStr">
+        <is>
+          <t>ik@veripark.com, kariyer@veripark.com, career@veripark.com, cv@veripark.com</t>
+        </is>
+      </c>
+      <c r="E98" s="2" t="inlineStr">
+        <is>
+          <t>Bankacılık yazılımı</t>
+        </is>
+      </c>
+      <c r="F98" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G98" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
+        </is>
+      </c>
+      <c r="H98" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft 365</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="inlineStr">
+        <is>
+          <t>Verisoft</t>
+        </is>
+      </c>
+      <c r="B99" s="2" t="inlineStr">
+        <is>
+          <t>https://verisoft.com</t>
+        </is>
+      </c>
+      <c r="C99" s="2" t="inlineStr"/>
+      <c r="D99" s="3" t="inlineStr">
+        <is>
+          <t>ik@verisoft.com, kariyer@verisoft.com, career@verisoft.com, cv@verisoft.com</t>
+        </is>
+      </c>
+      <c r="E99" s="2" t="inlineStr"/>
+      <c r="F99" s="2" t="inlineStr">
+        <is>
+          <t>Kullanıcı listesi (05.08.2026 - 2. parti)</t>
+        </is>
+      </c>
+      <c r="G99" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
+        </is>
+      </c>
+      <c r="H99" s="2" t="inlineStr">
+        <is>
+          <t>Google Workspace</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="inlineStr">
+        <is>
+          <t>Virgosol</t>
+        </is>
+      </c>
+      <c r="B100" s="2" t="inlineStr">
+        <is>
+          <t>https://virgosol.com</t>
+        </is>
+      </c>
+      <c r="C100" s="2" t="inlineStr"/>
+      <c r="D100" s="3" t="inlineStr">
+        <is>
+          <t>ik@virgosol.com, kariyer@virgosol.com, career@virgosol.com, cv@virgosol.com</t>
+        </is>
+      </c>
+      <c r="E100" s="2" t="inlineStr">
+        <is>
+          <t>Yazılım geliştirme</t>
+        </is>
+      </c>
+      <c r="F100" s="2" t="inlineStr">
+        <is>
+          <t>Kullanıcı listesi (05.08.2026)</t>
+        </is>
+      </c>
+      <c r="G100" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
+        </is>
+      </c>
+      <c r="H100" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft 365</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="2" t="inlineStr">
+        <is>
+          <t>Vispera</t>
+        </is>
+      </c>
+      <c r="B101" s="2" t="inlineStr">
+        <is>
+          <t>https://vispera.co</t>
+        </is>
+      </c>
+      <c r="C101" s="2" t="inlineStr"/>
+      <c r="D101" s="3" t="inlineStr">
+        <is>
+          <t>ik@vispera.co, kariyer@vispera.co, career@vispera.co, cv@vispera.co</t>
+        </is>
+      </c>
+      <c r="E101" s="2" t="inlineStr">
+        <is>
+          <t>Yapay zeka / görüntü işleme</t>
+        </is>
+      </c>
+      <c r="F101" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G101" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
+        </is>
+      </c>
+      <c r="H101" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft 365</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t>VoltLines</t>
+        </is>
+      </c>
+      <c r="B102" s="2" t="inlineStr">
+        <is>
+          <t>https://voltlines.com</t>
+        </is>
+      </c>
+      <c r="C102" s="2" t="inlineStr"/>
+      <c r="D102" s="3" t="inlineStr">
+        <is>
+          <t>ik@voltlines.com, kariyer@voltlines.com, career@voltlines.com, cv@voltlines.com</t>
+        </is>
+      </c>
+      <c r="E102" s="2" t="inlineStr">
+        <is>
+          <t>Kurumsal ulaşım teknolojisi</t>
+        </is>
+      </c>
+      <c r="F102" s="2" t="inlineStr">
+        <is>
+          <t>Kullanıcı listesi (05.08.2026)</t>
+        </is>
+      </c>
+      <c r="G102" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
+        </is>
+      </c>
+      <c r="H102" s="2" t="inlineStr">
+        <is>
+          <t>Google Workspace</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="2" t="inlineStr">
+        <is>
+          <t>Workcube</t>
+        </is>
+      </c>
+      <c r="B103" s="2" t="inlineStr">
+        <is>
+          <t>https://www.workcube.com</t>
+        </is>
+      </c>
+      <c r="C103" s="2" t="inlineStr"/>
+      <c r="D103" s="3" t="inlineStr">
+        <is>
+          <t>ik@workcube.com, kariyer@workcube.com, career@workcube.com, cv@workcube.com</t>
+        </is>
+      </c>
+      <c r="E103" s="2" t="inlineStr">
+        <is>
+          <t>Kurumsal yazılım / ERP</t>
+        </is>
+      </c>
+      <c r="F103" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G103" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
+        </is>
+      </c>
+      <c r="H103" s="2" t="inlineStr">
+        <is>
+          <t>Google Workspace</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="2" t="inlineStr">
+        <is>
+          <t>Yemeksepeti</t>
+        </is>
+      </c>
+      <c r="B104" s="2" t="inlineStr">
+        <is>
+          <t>https://www.yemeksepeti.com</t>
+        </is>
+      </c>
+      <c r="C104" s="2" t="inlineStr"/>
+      <c r="D104" s="3" t="inlineStr">
+        <is>
           <t>ik@yemeksepeti.com, kariyer@yemeksepeti.com, career@yemeksepeti.com, cv@yemeksepeti.com</t>
         </is>
       </c>
-      <c r="E94" s="2" t="inlineStr">
+      <c r="E104" s="2" t="inlineStr">
         <is>
           <t>Online yemek siparişi</t>
         </is>
       </c>
-      <c r="F94" s="2" t="inlineStr">
-        <is>
-          <t>Ön liste (doğrulanmadı)</t>
-        </is>
-      </c>
-      <c r="G94" s="3" t="inlineStr">
-        <is>
-          <t>üretildi – doğrulanmadı</t>
-        </is>
-      </c>
-      <c r="H94" s="2" t="inlineStr">
+      <c r="F104" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G104" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
+        </is>
+      </c>
+      <c r="H104" s="2" t="inlineStr">
         <is>
           <t>Google Workspace</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H94"/>
+  <autoFilter ref="A1:H104"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Üçüncü parti: 9 firma eklendi
dataliva.com, applogist.com, odeontechnology.com, moneypay.com.tr,
argela.com.tr, quicksigorta.com, pozitiftech.com, inveon.com, deloitte.com
eklendi; dokuzunun da MX kaydı doğrulandı. epigra.com ikinci partide
eklendiği için tekilleştirildi.

Toplam 112 firma, 111'inin alan adı mail kabul ediyor.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016m9M3fsJ1qn42BpGV3myHC
</commit_message>
<xml_diff>
--- a/istanbul_yazilim_sirketleri.xlsx
+++ b/istanbul_yazilim_sirketleri.xlsx
@@ -11,7 +11,7 @@
     <sheet name="OKUBENI" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Şirketler'!$A$1:$H$104</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Şirketler'!$A$1:$H$113</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H104"/>
+  <dimension ref="A1:H113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -590,28 +590,28 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Armut</t>
+          <t>Applogist</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>https://www.armut.com</t>
+          <t>https://www.applogist.com</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr"/>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>ik@armut.com, kariyer@armut.com, career@armut.com, cv@armut.com</t>
+          <t>ik@applogist.com, kariyer@applogist.com, career@applogist.com, cv@applogist.com</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Hizmet pazaryeri</t>
+          <t>Mobil uygulama geliştirme</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Kullanıcı listesi (05.08.2026 - 3. parti)</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
@@ -621,31 +621,35 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Google Workspace</t>
+          <t>Microsoft 365</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>ATP Teknoloji</t>
+          <t>Argela</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>https://www.atptech.com</t>
+          <t>https://www.argela.com.tr</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr"/>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>ik@atptech.com, kariyer@atptech.com, career@atptech.com, cv@atptech.com</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr"/>
+          <t>ik@argela.com.tr, kariyer@argela.com.tr, career@argela.com.tr, cv@argela.com.tr</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Telekom yazılımı</t>
+        </is>
+      </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Kullanıcı listesi (05.08.2026)</t>
+          <t>Kullanıcı listesi (05.08.2026 - 3. parti)</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -655,31 +659,35 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>var</t>
+          <t>Microsoft 365</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>AVDCG</t>
+          <t>Armut</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>https://avdcg.com</t>
+          <t>https://www.armut.com</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr"/>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>ik@avdcg.com, kariyer@avdcg.com, career@avdcg.com, cv@avdcg.com</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr"/>
+          <t>ik@armut.com, kariyer@armut.com, career@armut.com, cv@armut.com</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Hizmet pazaryeri</t>
+        </is>
+      </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Kullanıcı listesi (05.08.2026)</t>
+          <t>Ön liste (doğrulanmadı)</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
@@ -689,35 +697,31 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Microsoft 365</t>
+          <t>Google Workspace</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Berqnet</t>
+          <t>ATP Teknoloji</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>https://www.berqnet.com</t>
+          <t>https://www.atptech.com</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr"/>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>ik@berqnet.com, kariyer@berqnet.com, career@berqnet.com, cv@berqnet.com</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>Siber güvenlik / güvenlik duvarı</t>
-        </is>
-      </c>
+          <t>ik@atptech.com, kariyer@atptech.com, career@atptech.com, cv@atptech.com</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr"/>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Kullanıcı listesi (05.08.2026)</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
@@ -727,32 +731,28 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Google Workspace</t>
+          <t>var</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Bimser Çözüm</t>
+          <t>AVDCG</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>https://bimser.com</t>
+          <t>https://avdcg.com</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr"/>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>ik@bimser.com, kariyer@bimser.com, career@bimser.com, cv@bimser.com</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>Kurumsal yazılım (QDMS / eBA)</t>
-        </is>
-      </c>
+          <t>ik@avdcg.com, kariyer@avdcg.com, career@avdcg.com, cv@avdcg.com</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="2" t="inlineStr">
         <is>
           <t>Kullanıcı listesi (05.08.2026)</t>
@@ -772,23 +772,23 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>BiTaksi</t>
+          <t>Berqnet</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>https://bitaksi.com</t>
+          <t>https://www.berqnet.com</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr"/>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>ik@bitaksi.com, kariyer@bitaksi.com, career@bitaksi.com, cv@bitaksi.com</t>
+          <t>ik@berqnet.com, kariyer@berqnet.com, career@berqnet.com, cv@berqnet.com</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Mobilite / mobil uygulama</t>
+          <t>Siber güvenlik / güvenlik duvarı</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -810,28 +810,28 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Bitexen</t>
+          <t>Bimser Çözüm</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>https://www.bitexen.com</t>
+          <t>https://bimser.com</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr"/>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>ik@bitexen.com, kariyer@bitexen.com, career@bitexen.com, cv@bitexen.com</t>
+          <t>ik@bimser.com, kariyer@bimser.com, career@bimser.com, cv@bimser.com</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Kripto varlık platformu</t>
+          <t>Kurumsal yazılım (QDMS / eBA)</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Kullanıcı listesi (05.08.2026)</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr">
@@ -848,24 +848,28 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Blue Arf</t>
+          <t>BiTaksi</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>https://www.bluearf.com</t>
+          <t>https://bitaksi.com</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr"/>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>ik@bluearf.com, kariyer@bluearf.com, career@bluearf.com, cv@bluearf.com</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr"/>
+          <t>ik@bitaksi.com, kariyer@bitaksi.com, career@bitaksi.com, cv@bitaksi.com</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Mobilite / mobil uygulama</t>
+        </is>
+      </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Kullanıcı listesi (05.08.2026)</t>
+          <t>Ön liste (doğrulanmadı)</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
@@ -882,18 +886,18 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>BtcTurk</t>
+          <t>Bitexen</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>https://www.btcturk.com</t>
+          <t>https://www.bitexen.com</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr"/>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>ik@btcturk.com, kariyer@btcturk.com, career@btcturk.com, cv@btcturk.com</t>
+          <t>ik@bitexen.com, kariyer@bitexen.com, career@bitexen.com, cv@bitexen.com</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -913,25 +917,25 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>var</t>
+          <t>Microsoft 365</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Chippin</t>
+          <t>Blue Arf</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>https://chippin.com</t>
+          <t>https://www.bluearf.com</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr"/>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>ik@chippin.com, kariyer@chippin.com, career@chippin.com, cv@chippin.com</t>
+          <t>ik@bluearf.com, kariyer@bluearf.com, career@bluearf.com, cv@bluearf.com</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr"/>
@@ -947,35 +951,35 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>var</t>
+          <t>Google Workspace</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Codevo</t>
+          <t>BtcTurk</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>https://codevo.com.tr</t>
+          <t>https://www.btcturk.com</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr"/>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>ik@codevo.com.tr, kariyer@codevo.com.tr, career@codevo.com.tr, cv@codevo.com.tr</t>
+          <t>ik@btcturk.com, kariyer@btcturk.com, career@btcturk.com, cv@btcturk.com</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Yazılım geliştirme</t>
+          <t>Kripto varlık platformu</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Kullanıcı listesi (05.08.2026)</t>
+          <t>Ön liste (doğrulanmadı)</t>
         </is>
       </c>
       <c r="G14" s="3" t="inlineStr">
@@ -985,35 +989,31 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>Microsoft 365</t>
+          <t>var</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Codeway</t>
+          <t>Chippin</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>https://codeway.co</t>
+          <t>https://chippin.com</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr"/>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>ik@codeway.co, kariyer@codeway.co, career@codeway.co, cv@codeway.co</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>Mobil uygulama geliştirme</t>
-        </is>
-      </c>
+          <t>ik@chippin.com, kariyer@chippin.com, career@chippin.com, cv@chippin.com</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Kullanıcı listesi (05.08.2026)</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
@@ -1023,35 +1023,35 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>Google Workspace</t>
+          <t>var</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Colendi</t>
+          <t>Codevo</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>https://www.colendi.com</t>
+          <t>https://codevo.com.tr</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr"/>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>ik@colendi.com, kariyer@colendi.com, career@colendi.com, cv@colendi.com</t>
+          <t>ik@codevo.com.tr, kariyer@codevo.com.tr, career@codevo.com.tr, cv@codevo.com.tr</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Fintech / dijital bankacılık</t>
+          <t>Yazılım geliştirme</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Kullanıcı listesi (05.08.2026)</t>
         </is>
       </c>
       <c r="G16" s="3" t="inlineStr">
@@ -1061,30 +1061,30 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>Google Workspace</t>
+          <t>Microsoft 365</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Commencis</t>
+          <t>Codeway</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>https://www.commencis.com</t>
+          <t>https://codeway.co</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr"/>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>ik@commencis.com, kariyer@commencis.com, career@commencis.com, cv@commencis.com</t>
+          <t>ik@codeway.co, kariyer@codeway.co, career@codeway.co, cv@codeway.co</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Dijital ürün / yazılım geliştirme</t>
+          <t>Mobil uygulama geliştirme</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
@@ -1099,30 +1099,30 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>Microsoft 365</t>
+          <t>Google Workspace</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>CPM Yazılım</t>
+          <t>Colendi</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>https://www.cpm.com.tr</t>
+          <t>https://www.colendi.com</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr"/>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>ik@cpm.com.tr, kariyer@cpm.com.tr, career@cpm.com.tr, cv@cpm.com.tr</t>
+          <t>ik@colendi.com, kariyer@colendi.com, career@colendi.com, cv@colendi.com</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Sigortacılık yazılımı</t>
+          <t>Fintech / dijital bankacılık</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -1137,30 +1137,30 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>Microsoft 365</t>
+          <t>Google Workspace</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Craftgate</t>
+          <t>Commencis</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>https://craftgate.io</t>
+          <t>https://www.commencis.com</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr"/>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>ik@craftgate.io, kariyer@craftgate.io, career@craftgate.io, cv@craftgate.io</t>
+          <t>ik@commencis.com, kariyer@commencis.com, career@commencis.com, cv@commencis.com</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Fintech / ödeme altyapısı</t>
+          <t>Dijital ürün / yazılım geliştirme</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
@@ -1175,31 +1175,35 @@
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>Google Workspace</t>
+          <t>Microsoft 365</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>CRS Soft</t>
+          <t>CPM Yazılım</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>https://www.crssoft.com</t>
+          <t>https://www.cpm.com.tr</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr"/>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>ik@crssoft.com, kariyer@crssoft.com, career@crssoft.com, cv@crssoft.com</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr"/>
+          <t>ik@cpm.com.tr, kariyer@cpm.com.tr, career@cpm.com.tr, cv@cpm.com.tr</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Sigortacılık yazılımı</t>
+        </is>
+      </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Kullanıcı listesi (05.08.2026)</t>
+          <t>Ön liste (doğrulanmadı)</t>
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr">
@@ -1216,23 +1220,23 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Detaysoft</t>
+          <t>Craftgate</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>https://www.detaysoft.com</t>
+          <t>https://craftgate.io</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr"/>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>ik@detaysoft.com, kariyer@detaysoft.com, career@detaysoft.com, cv@detaysoft.com</t>
+          <t>ik@craftgate.io, kariyer@craftgate.io, career@craftgate.io, cv@craftgate.io</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>SAP danışmanlık / kurumsal yazılım</t>
+          <t>Fintech / ödeme altyapısı</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
@@ -1247,35 +1251,31 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>var</t>
+          <t>Google Workspace</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Digital Planet</t>
+          <t>CRS Soft</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>https://www.digitalplanet.com.tr</t>
+          <t>https://www.crssoft.com</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr"/>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>ik@digitalplanet.com.tr, kariyer@digitalplanet.com.tr, career@digitalplanet.com.tr, cv@digitalplanet.com.tr</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>e-Dönüşüm çözümleri</t>
-        </is>
-      </c>
+          <t>ik@crssoft.com, kariyer@crssoft.com, career@crssoft.com, cv@crssoft.com</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr"/>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Kullanıcı listesi (05.08.2026)</t>
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr">
@@ -1292,28 +1292,28 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Dijital Kurye</t>
+          <t>Dataliva</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>https://dijitalkurye.com.tr</t>
+          <t>https://www.dataliva.com</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr"/>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>ik@dijitalkurye.com.tr, kariyer@dijitalkurye.com.tr, career@dijitalkurye.com.tr, cv@dijitalkurye.com.tr</t>
+          <t>ik@dataliva.com, kariyer@dataliva.com, career@dataliva.com, cv@dataliva.com</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Dijital ajans</t>
+          <t>Veri analitiği / yapay zeka</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Kullanıcı listesi (05.08.2026)</t>
+          <t>Kullanıcı listesi (05.08.2026 - 3. parti)</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
@@ -1330,28 +1330,28 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Doğuş Teknoloji</t>
+          <t>Deloitte</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>https://www.d-teknoloji.com.tr</t>
+          <t>https://www.deloitte.com</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr"/>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>ik@d-teknoloji.com.tr, kariyer@d-teknoloji.com.tr, career@d-teknoloji.com.tr, cv@d-teknoloji.com.tr</t>
+          <t>ik@deloitte.com, kariyer@deloitte.com, career@deloitte.com, cv@deloitte.com</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>BT hizmetleri</t>
+          <t>Denetim / danışmanlık</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Kullanıcı listesi (05.08.2026 - 3. parti)</t>
         </is>
       </c>
       <c r="G24" s="3" t="inlineStr">
@@ -1361,30 +1361,30 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>Microsoft 365</t>
+          <t>var</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Dream Games</t>
+          <t>Detaysoft</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>https://www.dreamgames.com</t>
+          <t>https://www.detaysoft.com</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr"/>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>ik@dreamgames.com, kariyer@dreamgames.com, career@dreamgames.com, cv@dreamgames.com</t>
+          <t>ik@detaysoft.com, kariyer@detaysoft.com, career@detaysoft.com, cv@detaysoft.com</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Mobil oyun</t>
+          <t>SAP danışmanlık / kurumsal yazılım</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
@@ -1399,35 +1399,35 @@
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>Google Workspace</t>
+          <t>var</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Epigra</t>
+          <t>Digital Planet</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>https://epigra.com</t>
+          <t>https://www.digitalplanet.com.tr</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr"/>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>ik@epigra.com, kariyer@epigra.com, career@epigra.com, cv@epigra.com</t>
+          <t>ik@digitalplanet.com.tr, kariyer@digitalplanet.com.tr, career@digitalplanet.com.tr, cv@digitalplanet.com.tr</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Dijital ajans / web geliştirme</t>
+          <t>e-Dönüşüm çözümleri</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Kullanıcı listesi (05.08.2026 - 2. parti)</t>
+          <t>Ön liste (doğrulanmadı)</t>
         </is>
       </c>
       <c r="G26" s="3" t="inlineStr">
@@ -1437,35 +1437,35 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>Google Workspace</t>
+          <t>Microsoft 365</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Etiya</t>
+          <t>Dijital Kurye</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>https://www.etiya.com</t>
+          <t>https://dijitalkurye.com.tr</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr"/>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>ik@etiya.com, kariyer@etiya.com, career@etiya.com, cv@etiya.com</t>
+          <t>ik@dijitalkurye.com.tr, kariyer@dijitalkurye.com.tr, career@dijitalkurye.com.tr, cv@dijitalkurye.com.tr</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Telekom yazılımı / BSS</t>
+          <t>Dijital ajans</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Kullanıcı listesi (05.08.2026)</t>
         </is>
       </c>
       <c r="G27" s="3" t="inlineStr">
@@ -1482,23 +1482,23 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Experteam</t>
+          <t>Doğuş Teknoloji</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>https://www.experteam.com.tr</t>
+          <t>https://www.d-teknoloji.com.tr</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr"/>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>ik@experteam.com.tr, kariyer@experteam.com.tr, career@experteam.com.tr, cv@experteam.com.tr</t>
+          <t>ik@d-teknoloji.com.tr, kariyer@d-teknoloji.com.tr, career@d-teknoloji.com.tr, cv@d-teknoloji.com.tr</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>SAP danışmanlık</t>
+          <t>BT hizmetleri</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
@@ -1520,23 +1520,23 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Figopara</t>
+          <t>Dream Games</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>https://www.figopara.com</t>
+          <t>https://www.dreamgames.com</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr"/>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>ik@figopara.com, kariyer@figopara.com, career@figopara.com, cv@figopara.com</t>
+          <t>ik@dreamgames.com, kariyer@dreamgames.com, career@dreamgames.com, cv@dreamgames.com</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Fintech / tedarik zinciri finansmanı</t>
+          <t>Mobil oyun</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
@@ -1551,28 +1551,32 @@
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>Microsoft 365</t>
+          <t>Google Workspace</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Finago Tech</t>
+          <t>Epigra</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>https://finagotech.com.tr</t>
+          <t>https://epigra.com</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr"/>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>ik@finagotech.com.tr, kariyer@finagotech.com.tr, career@finagotech.com.tr, cv@finagotech.com.tr</t>
-        </is>
-      </c>
-      <c r="E30" s="2" t="inlineStr"/>
+          <t>ik@epigra.com, kariyer@epigra.com, career@epigra.com, cv@epigra.com</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>Dijital ajans / web geliştirme</t>
+        </is>
+      </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
           <t>Kullanıcı listesi (05.08.2026 - 2. parti)</t>
@@ -1585,30 +1589,30 @@
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>Microsoft 365</t>
+          <t>Google Workspace</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Getir</t>
+          <t>Etiya</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>https://getir.com</t>
+          <t>https://www.etiya.com</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr"/>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>ik@getir.com, kariyer@getir.com, career@getir.com, cv@getir.com</t>
+          <t>ik@etiya.com, kariyer@etiya.com, career@etiya.com, cv@etiya.com</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Hızlı ticaret / mobil uygulama</t>
+          <t>Telekom yazılımı / BSS</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
@@ -1623,30 +1627,30 @@
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>Google Workspace</t>
+          <t>Microsoft 365</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Gram Games</t>
+          <t>Experteam</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>https://www.gramgames.com</t>
+          <t>https://www.experteam.com.tr</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr"/>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>ik@gramgames.com, kariyer@gramgames.com, career@gramgames.com, cv@gramgames.com</t>
+          <t>ik@experteam.com.tr, kariyer@experteam.com.tr, career@experteam.com.tr, cv@experteam.com.tr</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Mobil oyun</t>
+          <t>SAP danışmanlık</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
@@ -1656,40 +1660,40 @@
       </c>
       <c r="G32" s="3" t="inlineStr">
         <is>
-          <t>üretildi – MX YOK, kesin bounce eder</t>
-        </is>
-      </c>
-      <c r="H32" s="3" t="inlineStr">
-        <is>
-          <t>MX YOK (MX kaydı yok)</t>
+          <t>üretildi – doğrulanmadı</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft 365</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Grid Studio</t>
+          <t>Figopara</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>https://gridstudio.ai</t>
+          <t>https://www.figopara.com</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr"/>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>ik@gridstudio.ai, kariyer@gridstudio.ai, career@gridstudio.ai, cv@gridstudio.ai</t>
+          <t>ik@figopara.com, kariyer@figopara.com, career@figopara.com, cv@figopara.com</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>Yapay zeka</t>
+          <t>Fintech / tedarik zinciri finansmanı</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>Kullanıcı listesi (05.08.2026)</t>
+          <t>Ön liste (doğrulanmadı)</t>
         </is>
       </c>
       <c r="G33" s="3" t="inlineStr">
@@ -1699,35 +1703,31 @@
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>Google Workspace</t>
+          <t>Microsoft 365</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Hepsiburada</t>
+          <t>Finago Tech</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>https://www.hepsiburada.com</t>
+          <t>https://finagotech.com.tr</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr"/>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>ik@hepsiburada.com, kariyer@hepsiburada.com, career@hepsiburada.com, cv@hepsiburada.com</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="inlineStr">
-        <is>
-          <t>E-ticaret platformu</t>
-        </is>
-      </c>
+          <t>ik@finagotech.com.tr, kariyer@finagotech.com.tr, career@finagotech.com.tr, cv@finagotech.com.tr</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr"/>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Kullanıcı listesi (05.08.2026 - 2. parti)</t>
         </is>
       </c>
       <c r="G34" s="3" t="inlineStr">
@@ -1737,35 +1737,35 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>Google Workspace</t>
+          <t>Microsoft 365</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>HireFeed</t>
+          <t>Getir</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>https://www.hirefeed.co.in</t>
+          <t>https://getir.com</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr"/>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>ik@hirefeed.co.in, kariyer@hirefeed.co.in, career@hirefeed.co.in, cv@hirefeed.co.in</t>
+          <t>ik@getir.com, kariyer@getir.com, career@getir.com, cv@getir.com</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>İK teknolojileri</t>
+          <t>Hızlı ticaret / mobil uygulama</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>Kullanıcı listesi (05.08.2026)</t>
+          <t>Ön liste (doğrulanmadı)</t>
         </is>
       </c>
       <c r="G35" s="3" t="inlineStr">
@@ -1775,30 +1775,30 @@
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>var</t>
+          <t>Google Workspace</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>IAS - Canias ERP</t>
+          <t>Gram Games</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>https://www.caniaserp.com</t>
+          <t>https://www.gramgames.com</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr"/>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>ik@caniaserp.com, kariyer@caniaserp.com, career@caniaserp.com, cv@caniaserp.com</t>
+          <t>ik@gramgames.com, kariyer@gramgames.com, career@gramgames.com, cv@gramgames.com</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>ERP yazılımı</t>
+          <t>Mobil oyun</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
@@ -1808,40 +1808,40 @@
       </c>
       <c r="G36" s="3" t="inlineStr">
         <is>
-          <t>üretildi – doğrulanmadı</t>
-        </is>
-      </c>
-      <c r="H36" s="2" t="inlineStr">
-        <is>
-          <t>var</t>
+          <t>üretildi – MX YOK, kesin bounce eder</t>
+        </is>
+      </c>
+      <c r="H36" s="3" t="inlineStr">
+        <is>
+          <t>MX YOK (MX kaydı yok)</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>IdeaSoft</t>
+          <t>Grid Studio</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>https://www.ideasoft.com.tr</t>
+          <t>https://gridstudio.ai</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr"/>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>ik@ideasoft.com.tr, kariyer@ideasoft.com.tr, career@ideasoft.com.tr, cv@ideasoft.com.tr</t>
+          <t>ik@gridstudio.ai, kariyer@gridstudio.ai, career@gridstudio.ai, cv@gridstudio.ai</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>E-ticaret altyapı yazılımı</t>
+          <t>Yapay zeka</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Kullanıcı listesi (05.08.2026)</t>
         </is>
       </c>
       <c r="G37" s="3" t="inlineStr">
@@ -1858,23 +1858,23 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>ininal</t>
+          <t>Hepsiburada</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>https://www.ininal.com</t>
+          <t>https://www.hepsiburada.com</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr"/>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>ik@ininal.com, kariyer@ininal.com, career@ininal.com, cv@ininal.com</t>
+          <t>ik@hepsiburada.com, kariyer@hepsiburada.com, career@hepsiburada.com, cv@hepsiburada.com</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Fintech / ön ödemeli kart</t>
+          <t>E-ticaret platformu</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
@@ -1889,35 +1889,35 @@
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>Microsoft 365</t>
+          <t>Google Workspace</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Innova Bilişim</t>
+          <t>HireFeed</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>https://www.innova.com.tr</t>
+          <t>https://www.hirefeed.co.in</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr"/>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>ik@innova.com.tr, kariyer@innova.com.tr, career@innova.com.tr, cv@innova.com.tr</t>
+          <t>ik@hirefeed.co.in, kariyer@hirefeed.co.in, career@hirefeed.co.in, cv@hirefeed.co.in</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>BT çözümleri / sistem entegrasyonu</t>
+          <t>İK teknolojileri</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Kullanıcı listesi (05.08.2026)</t>
         </is>
       </c>
       <c r="G39" s="3" t="inlineStr">
@@ -1934,23 +1934,23 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Insider</t>
+          <t>IAS - Canias ERP</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>https://useinsider.com</t>
+          <t>https://www.caniaserp.com</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr"/>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>ik@useinsider.com, kariyer@useinsider.com, career@useinsider.com, cv@useinsider.com</t>
+          <t>ik@caniaserp.com, kariyer@caniaserp.com, career@caniaserp.com, cv@caniaserp.com</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Pazarlama teknolojileri / SaaS</t>
+          <t>ERP yazılımı</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
@@ -1972,23 +1972,23 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Intertech</t>
+          <t>IdeaSoft</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>https://www.intertech.com.tr</t>
+          <t>https://www.ideasoft.com.tr</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr"/>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>ik@intertech.com.tr, kariyer@intertech.com.tr, career@intertech.com.tr, cv@intertech.com.tr</t>
+          <t>ik@ideasoft.com.tr, kariyer@ideasoft.com.tr, career@ideasoft.com.tr, cv@ideasoft.com.tr</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Bankacılık teknolojileri</t>
+          <t>E-ticaret altyapı yazılımı</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
@@ -2003,30 +2003,30 @@
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>var</t>
+          <t>Google Workspace</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>iyzico</t>
+          <t>ininal</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>https://www.iyzico.com</t>
+          <t>https://www.ininal.com</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr"/>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>ik@iyzico.com, kariyer@iyzico.com, career@iyzico.com, cv@iyzico.com</t>
+          <t>ik@ininal.com, kariyer@ininal.com, career@ininal.com, cv@ininal.com</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Fintech / ödeme sistemleri</t>
+          <t>Fintech / ön ödemeli kart</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
@@ -2048,23 +2048,23 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>İzibiz</t>
+          <t>Innova Bilişim</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>https://www.izibiz.com.tr</t>
+          <t>https://www.innova.com.tr</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr"/>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>ik@izibiz.com.tr, kariyer@izibiz.com.tr, career@izibiz.com.tr, cv@izibiz.com.tr</t>
+          <t>ik@innova.com.tr, kariyer@innova.com.tr, career@innova.com.tr, cv@innova.com.tr</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>e-Fatura / e-dönüşüm</t>
+          <t>BT çözümleri / sistem entegrasyonu</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
@@ -2079,30 +2079,30 @@
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>Microsoft 365</t>
+          <t>var</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Kariyer.net</t>
+          <t>Insider</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>https://www.kariyer.net</t>
+          <t>https://useinsider.com</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr"/>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>ik@kariyer.net, kariyer@kariyer.net, career@kariyer.net, cv@kariyer.net</t>
+          <t>ik@useinsider.com, kariyer@useinsider.com, career@useinsider.com, cv@useinsider.com</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>İK teknolojileri</t>
+          <t>Pazarlama teknolojileri / SaaS</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
@@ -2117,30 +2117,30 @@
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>Microsoft 365</t>
+          <t>var</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>KoçSistem</t>
+          <t>Intertech</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>https://www.kocsistem.com.tr</t>
+          <t>https://www.intertech.com.tr</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr"/>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>ik@kocsistem.com.tr, kariyer@kocsistem.com.tr, career@kocsistem.com.tr, cv@kocsistem.com.tr</t>
+          <t>ik@intertech.com.tr, kariyer@intertech.com.tr, career@intertech.com.tr, cv@intertech.com.tr</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>BT hizmetleri / sistem entegrasyonu</t>
+          <t>Bankacılık teknolojileri</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
@@ -2162,28 +2162,28 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Kron Technologies</t>
+          <t>Inveon</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>https://krontech.com</t>
+          <t>https://www.inveon.com</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr"/>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>ik@krontech.com, kariyer@krontech.com, career@krontech.com, cv@krontech.com</t>
+          <t>ik@inveon.com, kariyer@inveon.com, career@inveon.com, cv@inveon.com</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Siber güvenlik / erişim yönetimi</t>
+          <t>E-ticaret yazılımı</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Kullanıcı listesi (05.08.2026 - 3. parti)</t>
         </is>
       </c>
       <c r="G46" s="3" t="inlineStr">
@@ -2193,30 +2193,30 @@
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>Microsoft 365</t>
+          <t>Google Workspace</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>Link Bilgisayar</t>
+          <t>iyzico</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkbilgisayar.com.tr</t>
+          <t>https://www.iyzico.com</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr"/>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>ik@linkbilgisayar.com.tr, kariyer@linkbilgisayar.com.tr, career@linkbilgisayar.com.tr, cv@linkbilgisayar.com.tr</t>
+          <t>ik@iyzico.com, kariyer@iyzico.com, career@iyzico.com, cv@iyzico.com</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>Ticari yazılım</t>
+          <t>Fintech / ödeme sistemleri</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
@@ -2238,28 +2238,28 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Loodos</t>
+          <t>İzibiz</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>https://loodos.com</t>
+          <t>https://www.izibiz.com.tr</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr"/>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>ik@loodos.com, kariyer@loodos.com, career@loodos.com, cv@loodos.com</t>
+          <t>ik@izibiz.com.tr, kariyer@izibiz.com.tr, career@izibiz.com.tr, cv@izibiz.com.tr</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>Mobil uygulama geliştirme</t>
+          <t>e-Fatura / e-dönüşüm</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>Kullanıcı listesi (05.08.2026)</t>
+          <t>Ön liste (doğrulanmadı)</t>
         </is>
       </c>
       <c r="G48" s="3" t="inlineStr">
@@ -2269,35 +2269,35 @@
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>Google Workspace</t>
+          <t>Microsoft 365</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>Lyrebird Studio</t>
+          <t>Kariyer.net</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>https://www.lyrebirdstudio.net</t>
+          <t>https://www.kariyer.net</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr"/>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>ik@lyrebirdstudio.net, kariyer@lyrebirdstudio.net, career@lyrebirdstudio.net, cv@lyrebirdstudio.net</t>
+          <t>ik@kariyer.net, kariyer@kariyer.net, career@kariyer.net, cv@kariyer.net</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>Mobil uygulama / foto düzenleme</t>
+          <t>İK teknolojileri</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>Kullanıcı listesi (05.08.2026)</t>
+          <t>Ön liste (doğrulanmadı)</t>
         </is>
       </c>
       <c r="G49" s="3" t="inlineStr">
@@ -2307,30 +2307,30 @@
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>Google Workspace</t>
+          <t>Microsoft 365</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Martı</t>
+          <t>KoçSistem</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>https://www.marti.tech</t>
+          <t>https://www.kocsistem.com.tr</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr"/>
       <c r="D50" s="3" t="inlineStr">
         <is>
-          <t>ik@marti.tech, kariyer@marti.tech, career@marti.tech, cv@marti.tech</t>
+          <t>ik@kocsistem.com.tr, kariyer@kocsistem.com.tr, career@kocsistem.com.tr, cv@kocsistem.com.tr</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>Mobilite teknolojileri</t>
+          <t>BT hizmetleri / sistem entegrasyonu</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
@@ -2352,24 +2352,28 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>Mee Apps</t>
+          <t>Kron Technologies</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>https://meeapps.com.tr</t>
+          <t>https://krontech.com</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr"/>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>ik@meeapps.com.tr, kariyer@meeapps.com.tr, career@meeapps.com.tr, cv@meeapps.com.tr</t>
-        </is>
-      </c>
-      <c r="E51" s="2" t="inlineStr"/>
+          <t>ik@krontech.com, kariyer@krontech.com, career@krontech.com, cv@krontech.com</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>Siber güvenlik / erişim yönetimi</t>
+        </is>
+      </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>Kullanıcı listesi (05.08.2026 - 2. parti)</t>
+          <t>Ön liste (doğrulanmadı)</t>
         </is>
       </c>
       <c r="G51" s="3" t="inlineStr">
@@ -2379,30 +2383,30 @@
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>Google Workspace</t>
+          <t>Microsoft 365</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>Midas</t>
+          <t>Link Bilgisayar</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>https://www.getmidas.com</t>
+          <t>https://www.linkbilgisayar.com.tr</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr"/>
       <c r="D52" s="3" t="inlineStr">
         <is>
-          <t>ik@getmidas.com, kariyer@getmidas.com, career@getmidas.com, cv@getmidas.com</t>
+          <t>ik@linkbilgisayar.com.tr, kariyer@linkbilgisayar.com.tr, career@linkbilgisayar.com.tr, cv@linkbilgisayar.com.tr</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>Fintech / yatırım platformu</t>
+          <t>Ticari yazılım</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
@@ -2417,35 +2421,35 @@
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>var</t>
+          <t>Microsoft 365</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>Mikro Yazılım</t>
+          <t>Loodos</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>https://www.mikro.com.tr</t>
+          <t>https://loodos.com</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr"/>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>ik@mikro.com.tr, kariyer@mikro.com.tr, career@mikro.com.tr, cv@mikro.com.tr</t>
+          <t>ik@loodos.com, kariyer@loodos.com, career@loodos.com, cv@loodos.com</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>Muhasebe / ERP yazılımı</t>
+          <t>Mobil uygulama geliştirme</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Kullanıcı listesi (05.08.2026)</t>
         </is>
       </c>
       <c r="G53" s="3" t="inlineStr">
@@ -2455,35 +2459,35 @@
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
-          <t>var</t>
+          <t>Google Workspace</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>Mobiroller</t>
+          <t>Lyrebird Studio</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>https://www.mobiroller.com</t>
+          <t>https://www.lyrebirdstudio.net</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr"/>
       <c r="D54" s="3" t="inlineStr">
         <is>
-          <t>ik@mobiroller.com, kariyer@mobiroller.com, career@mobiroller.com, cv@mobiroller.com</t>
+          <t>ik@lyrebirdstudio.net, kariyer@lyrebirdstudio.net, career@lyrebirdstudio.net, cv@lyrebirdstudio.net</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>Mobil uygulama geliştirme platformu</t>
+          <t>Mobil uygulama / foto düzenleme</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Kullanıcı listesi (05.08.2026)</t>
         </is>
       </c>
       <c r="G54" s="3" t="inlineStr">
@@ -2500,23 +2504,23 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>Mobven</t>
+          <t>Martı</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>https://mobven.com</t>
+          <t>https://www.marti.tech</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr"/>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t>ik@mobven.com, kariyer@mobven.com, career@mobven.com, cv@mobven.com</t>
+          <t>ik@marti.tech, kariyer@marti.tech, career@marti.tech, cv@marti.tech</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>Mobil yazılım geliştirme</t>
+          <t>Mobilite teknolojileri</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
@@ -2531,35 +2535,31 @@
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>Google Workspace</t>
+          <t>var</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>Modanisa</t>
+          <t>Mee Apps</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>https://www.modanisa.com</t>
+          <t>https://meeapps.com.tr</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr"/>
       <c r="D56" s="3" t="inlineStr">
         <is>
-          <t>ik@modanisa.com, kariyer@modanisa.com, career@modanisa.com, cv@modanisa.com</t>
-        </is>
-      </c>
-      <c r="E56" s="2" t="inlineStr">
-        <is>
-          <t>E-ticaret</t>
-        </is>
-      </c>
+          <t>ik@meeapps.com.tr, kariyer@meeapps.com.tr, career@meeapps.com.tr, cv@meeapps.com.tr</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr"/>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Kullanıcı listesi (05.08.2026 - 2. parti)</t>
         </is>
       </c>
       <c r="G56" s="3" t="inlineStr">
@@ -2576,28 +2576,28 @@
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>Mono Dijital</t>
+          <t>Midas</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>https://monodijital.com</t>
+          <t>https://www.getmidas.com</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr"/>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t>ik@monodijital.com, kariyer@monodijital.com, career@monodijital.com, cv@monodijital.com</t>
+          <t>ik@getmidas.com, kariyer@getmidas.com, career@getmidas.com, cv@getmidas.com</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>Dijital ajans</t>
+          <t>Fintech / yatırım platformu</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>Kullanıcı listesi (05.08.2026)</t>
+          <t>Ön liste (doğrulanmadı)</t>
         </is>
       </c>
       <c r="G57" s="3" t="inlineStr">
@@ -2607,35 +2607,35 @@
       </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
-          <t>Yandex</t>
+          <t>var</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>Native Minds</t>
+          <t>Mikro Yazılım</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>https://nativeminds.ai</t>
+          <t>https://www.mikro.com.tr</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr"/>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t>ik@nativeminds.ai, kariyer@nativeminds.ai, career@nativeminds.ai, cv@nativeminds.ai</t>
+          <t>ik@mikro.com.tr, kariyer@mikro.com.tr, career@mikro.com.tr, cv@mikro.com.tr</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>Yapay zeka</t>
+          <t>Muhasebe / ERP yazılımı</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>Kullanıcı listesi (05.08.2026)</t>
+          <t>Ön liste (doğrulanmadı)</t>
         </is>
       </c>
       <c r="G58" s="3" t="inlineStr">
@@ -2645,30 +2645,30 @@
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>Google Workspace</t>
+          <t>var</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>Nebim</t>
+          <t>Mobiroller</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>https://www.nebim.com.tr</t>
+          <t>https://www.mobiroller.com</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr"/>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>ik@nebim.com.tr, kariyer@nebim.com.tr, career@nebim.com.tr, cv@nebim.com.tr</t>
+          <t>ik@mobiroller.com, kariyer@mobiroller.com, career@mobiroller.com, cv@mobiroller.com</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>Perakende ERP yazılımı</t>
+          <t>Mobil uygulama geliştirme platformu</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
@@ -2690,28 +2690,28 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>Neon Apps</t>
+          <t>Mobven</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>https://neonapps.co</t>
+          <t>https://mobven.com</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr"/>
       <c r="D60" s="3" t="inlineStr">
         <is>
-          <t>ik@neonapps.co, kariyer@neonapps.co, career@neonapps.co, cv@neonapps.co</t>
+          <t>ik@mobven.com, kariyer@mobven.com, career@mobven.com, cv@mobven.com</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>Mobil uygulama geliştirme</t>
+          <t>Mobil yazılım geliştirme</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>Kullanıcı listesi (05.08.2026)</t>
+          <t>Ön liste (doğrulanmadı)</t>
         </is>
       </c>
       <c r="G60" s="3" t="inlineStr">
@@ -2728,24 +2728,28 @@
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>Neova</t>
+          <t>Modanisa</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>https://neova.com.tr</t>
+          <t>https://www.modanisa.com</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr"/>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t>ik@neova.com.tr, kariyer@neova.com.tr, career@neova.com.tr, cv@neova.com.tr</t>
-        </is>
-      </c>
-      <c r="E61" s="2" t="inlineStr"/>
+          <t>ik@modanisa.com, kariyer@modanisa.com, career@modanisa.com, cv@modanisa.com</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>E-ticaret</t>
+        </is>
+      </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>Kullanıcı listesi (05.08.2026 - 2. parti)</t>
+          <t>Ön liste (doğrulanmadı)</t>
         </is>
       </c>
       <c r="G61" s="3" t="inlineStr">
@@ -2755,35 +2759,35 @@
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
-          <t>var</t>
+          <t>Google Workspace</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>Netaş</t>
+          <t>MoneyPay</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>https://www.netas.com.tr</t>
+          <t>https://www.moneypay.com.tr</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr"/>
       <c r="D62" s="3" t="inlineStr">
         <is>
-          <t>ik@netas.com.tr, kariyer@netas.com.tr, career@netas.com.tr, cv@netas.com.tr</t>
+          <t>ik@moneypay.com.tr, kariyer@moneypay.com.tr, career@moneypay.com.tr, cv@moneypay.com.tr</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>Telekom ve yazılım çözümleri</t>
+          <t>Fintech / ödeme sistemleri</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Kullanıcı listesi (05.08.2026 - 3. parti)</t>
         </is>
       </c>
       <c r="G62" s="3" t="inlineStr">
@@ -2800,23 +2804,23 @@
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>NGaming</t>
+          <t>Mono Dijital</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>https://ngaming.com</t>
+          <t>https://monodijital.com</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr"/>
       <c r="D63" s="3" t="inlineStr">
         <is>
-          <t>ik@ngaming.com, kariyer@ngaming.com, career@ngaming.com, cv@ngaming.com</t>
+          <t>ik@monodijital.com, kariyer@monodijital.com, career@monodijital.com, cv@monodijital.com</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>Oyun</t>
+          <t>Dijital ajans</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
@@ -2831,28 +2835,32 @@
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
-          <t>Microsoft 365</t>
+          <t>Yandex</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>Oak Technology</t>
+          <t>Native Minds</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>https://oak.technology</t>
+          <t>https://nativeminds.ai</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr"/>
       <c r="D64" s="3" t="inlineStr">
         <is>
-          <t>ik@oak.technology, kariyer@oak.technology, career@oak.technology, cv@oak.technology</t>
-        </is>
-      </c>
-      <c r="E64" s="2" t="inlineStr"/>
+          <t>ik@nativeminds.ai, kariyer@nativeminds.ai, career@nativeminds.ai, cv@nativeminds.ai</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>Yapay zeka</t>
+        </is>
+      </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
           <t>Kullanıcı listesi (05.08.2026)</t>
@@ -2865,30 +2873,30 @@
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t>var</t>
+          <t>Google Workspace</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>OBSS</t>
+          <t>Nebim</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>https://obss.tech</t>
+          <t>https://www.nebim.com.tr</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr"/>
       <c r="D65" s="3" t="inlineStr">
         <is>
-          <t>ik@obss.tech, kariyer@obss.tech, career@obss.tech, cv@obss.tech</t>
+          <t>ik@nebim.com.tr, kariyer@nebim.com.tr, career@nebim.com.tr, cv@nebim.com.tr</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>Yazılım geliştirme / danışmanlık</t>
+          <t>Perakende ERP yazılımı</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
@@ -2910,28 +2918,28 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>Papara</t>
+          <t>Neon Apps</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>https://www.papara.com</t>
+          <t>https://neonapps.co</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr"/>
       <c r="D66" s="3" t="inlineStr">
         <is>
-          <t>ik@papara.com, kariyer@papara.com, career@papara.com, cv@papara.com</t>
+          <t>ik@neonapps.co, kariyer@neonapps.co, career@neonapps.co, cv@neonapps.co</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>Fintech / dijital cüzdan</t>
+          <t>Mobil uygulama geliştirme</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Kullanıcı listesi (05.08.2026)</t>
         </is>
       </c>
       <c r="G66" s="3" t="inlineStr">
@@ -2941,35 +2949,31 @@
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
-          <t>Microsoft 365</t>
+          <t>Google Workspace</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>Param</t>
+          <t>Neova</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>https://www.param.com.tr</t>
+          <t>https://neova.com.tr</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr"/>
       <c r="D67" s="3" t="inlineStr">
         <is>
-          <t>ik@param.com.tr, kariyer@param.com.tr, career@param.com.tr, cv@param.com.tr</t>
-        </is>
-      </c>
-      <c r="E67" s="2" t="inlineStr">
-        <is>
-          <t>Fintech / ödeme sistemleri</t>
-        </is>
-      </c>
+          <t>ik@neova.com.tr, kariyer@neova.com.tr, career@neova.com.tr, cv@neova.com.tr</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="inlineStr"/>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Kullanıcı listesi (05.08.2026 - 2. parti)</t>
         </is>
       </c>
       <c r="G67" s="3" t="inlineStr">
@@ -2979,30 +2983,30 @@
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
-          <t>Google Workspace</t>
+          <t>var</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>Paribu</t>
+          <t>Netaş</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>https://www.paribu.com</t>
+          <t>https://www.netas.com.tr</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr"/>
       <c r="D68" s="3" t="inlineStr">
         <is>
-          <t>ik@paribu.com, kariyer@paribu.com, career@paribu.com, cv@paribu.com</t>
+          <t>ik@netas.com.tr, kariyer@netas.com.tr, career@netas.com.tr, cv@netas.com.tr</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>Kripto varlık platformu</t>
+          <t>Telekom ve yazılım çözümleri</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
@@ -3017,35 +3021,35 @@
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
-          <t>Google Workspace</t>
+          <t>Microsoft 365</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>PayCore</t>
+          <t>NGaming</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>https://www.paycore.com</t>
+          <t>https://ngaming.com</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr"/>
       <c r="D69" s="3" t="inlineStr">
         <is>
-          <t>ik@paycore.com, kariyer@paycore.com, career@paycore.com, cv@paycore.com</t>
+          <t>ik@ngaming.com, kariyer@ngaming.com, career@ngaming.com, cv@ngaming.com</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>Fintech / kart teknolojileri</t>
+          <t>Oyun</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Kullanıcı listesi (05.08.2026)</t>
         </is>
       </c>
       <c r="G69" s="3" t="inlineStr">
@@ -3062,24 +3066,24 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>Paymore</t>
+          <t>Oak Technology</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>https://paymore.com.tr</t>
+          <t>https://oak.technology</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr"/>
       <c r="D70" s="3" t="inlineStr">
         <is>
-          <t>ik@paymore.com.tr, kariyer@paymore.com.tr, career@paymore.com.tr, cv@paymore.com.tr</t>
+          <t>ik@oak.technology, kariyer@oak.technology, career@oak.technology, cv@oak.technology</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr"/>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>Kullanıcı listesi (05.08.2026 - 2. parti)</t>
+          <t>Kullanıcı listesi (05.08.2026)</t>
         </is>
       </c>
       <c r="G70" s="3" t="inlineStr">
@@ -3089,30 +3093,30 @@
       </c>
       <c r="H70" s="2" t="inlineStr">
         <is>
-          <t>Google Workspace</t>
+          <t>var</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>Peak Games</t>
+          <t>OBSS</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>https://www.peak.com</t>
+          <t>https://obss.tech</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr"/>
       <c r="D71" s="3" t="inlineStr">
         <is>
-          <t>ik@peak.com, kariyer@peak.com, career@peak.com, cv@peak.com</t>
+          <t>ik@obss.tech, kariyer@obss.tech, career@obss.tech, cv@obss.tech</t>
         </is>
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>Mobil oyun</t>
+          <t>Yazılım geliştirme / danışmanlık</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
@@ -3134,28 +3138,24 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>Platin Bilişim</t>
+          <t>Odeon Technology</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>https://www.platinbilisim.com.tr</t>
+          <t>https://www.odeontechnology.com</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr"/>
       <c r="D72" s="3" t="inlineStr">
         <is>
-          <t>ik@platinbilisim.com.tr, kariyer@platinbilisim.com.tr, career@platinbilisim.com.tr, cv@platinbilisim.com.tr</t>
-        </is>
-      </c>
-      <c r="E72" s="2" t="inlineStr">
-        <is>
-          <t>BT çözümleri / sistem entegrasyonu</t>
-        </is>
-      </c>
+          <t>ik@odeontechnology.com, kariyer@odeontechnology.com, career@odeontechnology.com, cv@odeontechnology.com</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="inlineStr"/>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Kullanıcı listesi (05.08.2026 - 3. parti)</t>
         </is>
       </c>
       <c r="G72" s="3" t="inlineStr">
@@ -3172,28 +3172,28 @@
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>Playable Factory</t>
+          <t>Papara</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>https://playablefactory.com</t>
+          <t>https://www.papara.com</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr"/>
       <c r="D73" s="3" t="inlineStr">
         <is>
-          <t>ik@playablefactory.com, kariyer@playablefactory.com, career@playablefactory.com, cv@playablefactory.com</t>
+          <t>ik@papara.com, kariyer@papara.com, career@papara.com, cv@papara.com</t>
         </is>
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>Oynanabilir reklam / oyun teknolojisi</t>
+          <t>Fintech / dijital cüzdan</t>
         </is>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>Kullanıcı listesi (05.08.2026)</t>
+          <t>Ön liste (doğrulanmadı)</t>
         </is>
       </c>
       <c r="G73" s="3" t="inlineStr">
@@ -3203,30 +3203,30 @@
       </c>
       <c r="H73" s="2" t="inlineStr">
         <is>
-          <t>Google Workspace</t>
+          <t>Microsoft 365</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>Protel</t>
+          <t>Param</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>https://www.protel.com.tr</t>
+          <t>https://www.param.com.tr</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr"/>
       <c r="D74" s="3" t="inlineStr">
         <is>
-          <t>ik@protel.com.tr, kariyer@protel.com.tr, career@protel.com.tr, cv@protel.com.tr</t>
+          <t>ik@param.com.tr, kariyer@param.com.tr, career@param.com.tr, cv@param.com.tr</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>Otel ve restoran yazılımı</t>
+          <t>Fintech / ödeme sistemleri</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
@@ -3248,23 +3248,23 @@
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>Related Digital</t>
+          <t>Paribu</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>https://www.relateddigital.com</t>
+          <t>https://www.paribu.com</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr"/>
       <c r="D75" s="3" t="inlineStr">
         <is>
-          <t>ik@relateddigital.com, kariyer@relateddigital.com, career@relateddigital.com, cv@relateddigital.com</t>
+          <t>ik@paribu.com, kariyer@paribu.com, career@paribu.com, cv@paribu.com</t>
         </is>
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>Pazarlama teknolojileri</t>
+          <t>Kripto varlık platformu</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
@@ -3279,35 +3279,35 @@
       </c>
       <c r="H75" s="2" t="inlineStr">
         <is>
-          <t>Microsoft 365</t>
+          <t>Google Workspace</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>Rentcarla</t>
+          <t>PayCore</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>https://rentcarla.com</t>
+          <t>https://www.paycore.com</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr"/>
       <c r="D76" s="3" t="inlineStr">
         <is>
-          <t>ik@rentcarla.com, kariyer@rentcarla.com, career@rentcarla.com, cv@rentcarla.com</t>
+          <t>ik@paycore.com, kariyer@paycore.com, career@paycore.com, cv@paycore.com</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>Araç kiralama platformu</t>
+          <t>Fintech / kart teknolojileri</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>Kullanıcı listesi (05.08.2026)</t>
+          <t>Ön liste (doğrulanmadı)</t>
         </is>
       </c>
       <c r="G76" s="3" t="inlineStr">
@@ -3317,35 +3317,31 @@
       </c>
       <c r="H76" s="2" t="inlineStr">
         <is>
-          <t>Google Workspace</t>
+          <t>Microsoft 365</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>Rollic Games</t>
+          <t>Paymore</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>https://www.rollicgames.com</t>
+          <t>https://paymore.com.tr</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr"/>
       <c r="D77" s="3" t="inlineStr">
         <is>
-          <t>ik@rollicgames.com, kariyer@rollicgames.com, career@rollicgames.com, cv@rollicgames.com</t>
-        </is>
-      </c>
-      <c r="E77" s="2" t="inlineStr">
-        <is>
-          <t>Mobil oyun</t>
-        </is>
-      </c>
+          <t>ik@paymore.com.tr, kariyer@paymore.com.tr, career@paymore.com.tr, cv@paymore.com.tr</t>
+        </is>
+      </c>
+      <c r="E77" s="2" t="inlineStr"/>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Kullanıcı listesi (05.08.2026 - 2. parti)</t>
         </is>
       </c>
       <c r="G77" s="3" t="inlineStr">
@@ -3362,23 +3358,23 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>Sabancı DX</t>
+          <t>Peak Games</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>https://www.sabancidx.com</t>
+          <t>https://www.peak.com</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr"/>
       <c r="D78" s="3" t="inlineStr">
         <is>
-          <t>ik@sabancidx.com, kariyer@sabancidx.com, career@sabancidx.com, cv@sabancidx.com</t>
+          <t>ik@peak.com, kariyer@peak.com, career@peak.com, cv@peak.com</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>Dijital teknoloji / veri</t>
+          <t>Mobil oyun</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
@@ -3393,30 +3389,30 @@
       </c>
       <c r="H78" s="2" t="inlineStr">
         <is>
-          <t>var</t>
+          <t>Google Workspace</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>Sahibinden.com</t>
+          <t>Platin Bilişim</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>https://www.sahibinden.com</t>
+          <t>https://www.platinbilisim.com.tr</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr"/>
       <c r="D79" s="3" t="inlineStr">
         <is>
-          <t>ik@sahibinden.com, kariyer@sahibinden.com, career@sahibinden.com, cv@sahibinden.com</t>
+          <t>ik@platinbilisim.com.tr, kariyer@platinbilisim.com.tr, career@platinbilisim.com.tr, cv@platinbilisim.com.tr</t>
         </is>
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>Online ilan platformu</t>
+          <t>BT çözümleri / sistem entegrasyonu</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr">
@@ -3438,28 +3434,28 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>Segmentify</t>
+          <t>Playable Factory</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>https://www.segmentify.com</t>
+          <t>https://playablefactory.com</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr"/>
       <c r="D80" s="3" t="inlineStr">
         <is>
-          <t>ik@segmentify.com, kariyer@segmentify.com, career@segmentify.com, cv@segmentify.com</t>
+          <t>ik@playablefactory.com, kariyer@playablefactory.com, career@playablefactory.com, cv@playablefactory.com</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>E-ticaret kişiselleştirme</t>
+          <t>Oynanabilir reklam / oyun teknolojisi</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Kullanıcı listesi (05.08.2026)</t>
         </is>
       </c>
       <c r="G80" s="3" t="inlineStr">
@@ -3476,24 +3472,28 @@
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>ServiceCore</t>
+          <t>Pozitif Teknoloji</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>https://servicecore.app</t>
+          <t>https://pozitiftech.com</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr"/>
       <c r="D81" s="3" t="inlineStr">
         <is>
-          <t>ik@servicecore.app, kariyer@servicecore.app, career@servicecore.app, cv@servicecore.app</t>
-        </is>
-      </c>
-      <c r="E81" s="2" t="inlineStr"/>
+          <t>ik@pozitiftech.com, kariyer@pozitiftech.com, career@pozitiftech.com, cv@pozitiftech.com</t>
+        </is>
+      </c>
+      <c r="E81" s="2" t="inlineStr">
+        <is>
+          <t>BT çözümleri</t>
+        </is>
+      </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>Kullanıcı listesi (05.08.2026 - 2. parti)</t>
+          <t>Kullanıcı listesi (05.08.2026 - 3. parti)</t>
         </is>
       </c>
       <c r="G81" s="3" t="inlineStr">
@@ -3503,30 +3503,30 @@
       </c>
       <c r="H81" s="2" t="inlineStr">
         <is>
-          <t>var</t>
+          <t>Microsoft 365</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>Setrow</t>
+          <t>Protel</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>https://setrow.com</t>
+          <t>https://www.protel.com.tr</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr"/>
       <c r="D82" s="3" t="inlineStr">
         <is>
-          <t>ik@setrow.com, kariyer@setrow.com, career@setrow.com, cv@setrow.com</t>
+          <t>ik@protel.com.tr, kariyer@protel.com.tr, career@protel.com.tr, cv@protel.com.tr</t>
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>E-posta pazarlama teknolojisi</t>
+          <t>Otel ve restoran yazılımı</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
@@ -3541,35 +3541,35 @@
       </c>
       <c r="H82" s="2" t="inlineStr">
         <is>
-          <t>Microsoft 365</t>
+          <t>Google Workspace</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>Seven Apps</t>
+          <t>Quick Sigorta</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>https://sevenapps.co</t>
+          <t>https://www.quicksigorta.com</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr"/>
       <c r="D83" s="3" t="inlineStr">
         <is>
-          <t>ik@sevenapps.co, kariyer@sevenapps.co, career@sevenapps.co, cv@sevenapps.co</t>
+          <t>ik@quicksigorta.com, kariyer@quicksigorta.com, career@quicksigorta.com, cv@quicksigorta.com</t>
         </is>
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>Mobil uygulama geliştirme</t>
+          <t>Sigorta</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>Kullanıcı listesi (05.08.2026)</t>
+          <t>Kullanıcı listesi (05.08.2026 - 3. parti)</t>
         </is>
       </c>
       <c r="G83" s="3" t="inlineStr">
@@ -3579,35 +3579,35 @@
       </c>
       <c r="H83" s="2" t="inlineStr">
         <is>
-          <t>Google Workspace</t>
+          <t>Microsoft 365</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>Shipday</t>
+          <t>Related Digital</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>https://shipday.com</t>
+          <t>https://www.relateddigital.com</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr"/>
       <c r="D84" s="3" t="inlineStr">
         <is>
-          <t>ik@shipday.com, kariyer@shipday.com, career@shipday.com, cv@shipday.com</t>
+          <t>ik@relateddigital.com, kariyer@relateddigital.com, career@relateddigital.com, cv@relateddigital.com</t>
         </is>
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>Teslimat yönetimi yazılımı</t>
+          <t>Pazarlama teknolojileri</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>Kullanıcı listesi (05.08.2026 - 2. parti)</t>
+          <t>Ön liste (doğrulanmadı)</t>
         </is>
       </c>
       <c r="G84" s="3" t="inlineStr">
@@ -3617,35 +3617,35 @@
       </c>
       <c r="H84" s="2" t="inlineStr">
         <is>
-          <t>Google Workspace</t>
+          <t>Microsoft 365</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>Sipay</t>
+          <t>Rentcarla</t>
         </is>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>https://www.sipay.com.tr</t>
+          <t>https://rentcarla.com</t>
         </is>
       </c>
       <c r="C85" s="2" t="inlineStr"/>
       <c r="D85" s="3" t="inlineStr">
         <is>
-          <t>ik@sipay.com.tr, kariyer@sipay.com.tr, career@sipay.com.tr, cv@sipay.com.tr</t>
+          <t>ik@rentcarla.com, kariyer@rentcarla.com, career@rentcarla.com, cv@rentcarla.com</t>
         </is>
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>Fintech / ödeme sistemleri</t>
+          <t>Araç kiralama platformu</t>
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Kullanıcı listesi (05.08.2026)</t>
         </is>
       </c>
       <c r="G85" s="3" t="inlineStr">
@@ -3655,30 +3655,30 @@
       </c>
       <c r="H85" s="2" t="inlineStr">
         <is>
-          <t>Microsoft 365</t>
+          <t>Google Workspace</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>Sistaş</t>
+          <t>Rollic Games</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>https://www.sistas.com.tr</t>
+          <t>https://www.rollicgames.com</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr"/>
       <c r="D86" s="3" t="inlineStr">
         <is>
-          <t>ik@sistas.com.tr, kariyer@sistas.com.tr, career@sistas.com.tr, cv@sistas.com.tr</t>
+          <t>ik@rollicgames.com, kariyer@rollicgames.com, career@rollicgames.com, cv@rollicgames.com</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>BT çözümleri</t>
+          <t>Mobil oyun</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">
@@ -3693,35 +3693,35 @@
       </c>
       <c r="H86" s="2" t="inlineStr">
         <is>
-          <t>var</t>
+          <t>Google Workspace</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>Slayz</t>
+          <t>Sabancı DX</t>
         </is>
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>https://slayz.app</t>
+          <t>https://www.sabancidx.com</t>
         </is>
       </c>
       <c r="C87" s="2" t="inlineStr"/>
       <c r="D87" s="3" t="inlineStr">
         <is>
-          <t>ik@slayz.app, kariyer@slayz.app, career@slayz.app, cv@slayz.app</t>
+          <t>ik@sabancidx.com, kariyer@sabancidx.com, career@sabancidx.com, cv@sabancidx.com</t>
         </is>
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>Mobil uygulama</t>
+          <t>Dijital teknoloji / veri</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>Kullanıcı listesi (05.08.2026)</t>
+          <t>Ön liste (doğrulanmadı)</t>
         </is>
       </c>
       <c r="G87" s="3" t="inlineStr">
@@ -3731,30 +3731,30 @@
       </c>
       <c r="H87" s="2" t="inlineStr">
         <is>
-          <t>Microsoft 365</t>
+          <t>var</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>Softtech</t>
+          <t>Sahibinden.com</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>https://www.softtech.com.tr</t>
+          <t>https://www.sahibinden.com</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr"/>
       <c r="D88" s="3" t="inlineStr">
         <is>
-          <t>ik@softtech.com.tr, kariyer@softtech.com.tr, career@softtech.com.tr, cv@softtech.com.tr</t>
+          <t>ik@sahibinden.com, kariyer@sahibinden.com, career@sahibinden.com, cv@sahibinden.com</t>
         </is>
       </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
-          <t>Bankacılık yazılımı</t>
+          <t>Online ilan platformu</t>
         </is>
       </c>
       <c r="F88" s="2" t="inlineStr">
@@ -3769,35 +3769,35 @@
       </c>
       <c r="H88" s="2" t="inlineStr">
         <is>
-          <t>var</t>
+          <t>Microsoft 365</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>Solvoyo</t>
+          <t>Segmentify</t>
         </is>
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>https://solvoyo.com</t>
+          <t>https://www.segmentify.com</t>
         </is>
       </c>
       <c r="C89" s="2" t="inlineStr"/>
       <c r="D89" s="3" t="inlineStr">
         <is>
-          <t>ik@solvoyo.com, kariyer@solvoyo.com, career@solvoyo.com, cv@solvoyo.com</t>
+          <t>ik@segmentify.com, kariyer@segmentify.com, career@segmentify.com, cv@segmentify.com</t>
         </is>
       </c>
       <c r="E89" s="2" t="inlineStr">
         <is>
-          <t>Tedarik zinciri planlama / yapay zeka</t>
+          <t>E-ticaret kişiselleştirme</t>
         </is>
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
-          <t>Kullanıcı listesi (05.08.2026 - 2. parti)</t>
+          <t>Ön liste (doğrulanmadı)</t>
         </is>
       </c>
       <c r="G89" s="3" t="inlineStr">
@@ -3814,28 +3814,24 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>Spyke Games</t>
+          <t>ServiceCore</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>https://www.spykegames.com</t>
+          <t>https://servicecore.app</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr"/>
       <c r="D90" s="3" t="inlineStr">
         <is>
-          <t>ik@spykegames.com, kariyer@spykegames.com, career@spykegames.com, cv@spykegames.com</t>
-        </is>
-      </c>
-      <c r="E90" s="2" t="inlineStr">
-        <is>
-          <t>Mobil oyun</t>
-        </is>
-      </c>
+          <t>ik@servicecore.app, kariyer@servicecore.app, career@servicecore.app, cv@servicecore.app</t>
+        </is>
+      </c>
+      <c r="E90" s="2" t="inlineStr"/>
       <c r="F90" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Kullanıcı listesi (05.08.2026 - 2. parti)</t>
         </is>
       </c>
       <c r="G90" s="3" t="inlineStr">
@@ -3845,30 +3841,30 @@
       </c>
       <c r="H90" s="2" t="inlineStr">
         <is>
-          <t>Google Workspace</t>
+          <t>var</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>T-Soft</t>
+          <t>Setrow</t>
         </is>
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>https://www.tsoft.com.tr</t>
+          <t>https://setrow.com</t>
         </is>
       </c>
       <c r="C91" s="2" t="inlineStr"/>
       <c r="D91" s="3" t="inlineStr">
         <is>
-          <t>ik@tsoft.com.tr, kariyer@tsoft.com.tr, career@tsoft.com.tr, cv@tsoft.com.tr</t>
+          <t>ik@setrow.com, kariyer@setrow.com, career@setrow.com, cv@setrow.com</t>
         </is>
       </c>
       <c r="E91" s="2" t="inlineStr">
         <is>
-          <t>E-ticaret yazılımı</t>
+          <t>E-posta pazarlama teknolojisi</t>
         </is>
       </c>
       <c r="F91" s="2" t="inlineStr">
@@ -3883,28 +3879,32 @@
       </c>
       <c r="H91" s="2" t="inlineStr">
         <is>
-          <t>var</t>
+          <t>Microsoft 365</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>TankX</t>
+          <t>Seven Apps</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>https://tankx.co</t>
+          <t>https://sevenapps.co</t>
         </is>
       </c>
       <c r="C92" s="2" t="inlineStr"/>
       <c r="D92" s="3" t="inlineStr">
         <is>
-          <t>ik@tankx.co, kariyer@tankx.co, career@tankx.co, cv@tankx.co</t>
-        </is>
-      </c>
-      <c r="E92" s="2" t="inlineStr"/>
+          <t>ik@sevenapps.co, kariyer@sevenapps.co, career@sevenapps.co, cv@sevenapps.co</t>
+        </is>
+      </c>
+      <c r="E92" s="2" t="inlineStr">
+        <is>
+          <t>Mobil uygulama geliştirme</t>
+        </is>
+      </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
           <t>Kullanıcı listesi (05.08.2026)</t>
@@ -3924,28 +3924,28 @@
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>Testinium</t>
+          <t>Shipday</t>
         </is>
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>https://testinium.com</t>
+          <t>https://shipday.com</t>
         </is>
       </c>
       <c r="C93" s="2" t="inlineStr"/>
       <c r="D93" s="3" t="inlineStr">
         <is>
-          <t>ik@testinium.com, kariyer@testinium.com, career@testinium.com, cv@testinium.com</t>
+          <t>ik@shipday.com, kariyer@shipday.com, career@shipday.com, cv@shipday.com</t>
         </is>
       </c>
       <c r="E93" s="2" t="inlineStr">
         <is>
-          <t>Test otomasyonu / yazılım kalite</t>
+          <t>Teslimat yönetimi yazılımı</t>
         </is>
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Kullanıcı listesi (05.08.2026 - 2. parti)</t>
         </is>
       </c>
       <c r="G93" s="3" t="inlineStr">
@@ -3955,30 +3955,30 @@
       </c>
       <c r="H93" s="2" t="inlineStr">
         <is>
-          <t>Microsoft 365</t>
+          <t>Google Workspace</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>Ticimax</t>
+          <t>Sipay</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>https://www.ticimax.com</t>
+          <t>https://www.sipay.com.tr</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr"/>
       <c r="D94" s="3" t="inlineStr">
         <is>
-          <t>ik@ticimax.com, kariyer@ticimax.com, career@ticimax.com, cv@ticimax.com</t>
+          <t>ik@sipay.com.tr, kariyer@sipay.com.tr, career@sipay.com.tr, cv@sipay.com.tr</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr">
         <is>
-          <t>E-ticaret altyapı yazılımı</t>
+          <t>Fintech / ödeme sistemleri</t>
         </is>
       </c>
       <c r="F94" s="2" t="inlineStr">
@@ -4000,23 +4000,23 @@
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>Trendyol</t>
+          <t>Sistaş</t>
         </is>
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>https://www.trendyol.com</t>
+          <t>https://www.sistas.com.tr</t>
         </is>
       </c>
       <c r="C95" s="2" t="inlineStr"/>
       <c r="D95" s="3" t="inlineStr">
         <is>
-          <t>ik@trendyol.com, kariyer@trendyol.com, career@trendyol.com, cv@trendyol.com</t>
+          <t>ik@sistas.com.tr, kariyer@sistas.com.tr, career@sistas.com.tr, cv@sistas.com.tr</t>
         </is>
       </c>
       <c r="E95" s="2" t="inlineStr">
         <is>
-          <t>E-ticaret platformu</t>
+          <t>BT çözümleri</t>
         </is>
       </c>
       <c r="F95" s="2" t="inlineStr">
@@ -4038,28 +4038,28 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>Uyumsoft</t>
+          <t>Slayz</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>https://www.uyumsoft.com.tr</t>
+          <t>https://slayz.app</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr"/>
       <c r="D96" s="3" t="inlineStr">
         <is>
-          <t>ik@uyumsoft.com.tr, kariyer@uyumsoft.com.tr, career@uyumsoft.com.tr, cv@uyumsoft.com.tr</t>
+          <t>ik@slayz.app, kariyer@slayz.app, career@slayz.app, cv@slayz.app</t>
         </is>
       </c>
       <c r="E96" s="2" t="inlineStr">
         <is>
-          <t>ERP / e-dönüşüm yazılımı</t>
+          <t>Mobil uygulama</t>
         </is>
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Kullanıcı listesi (05.08.2026)</t>
         </is>
       </c>
       <c r="G96" s="3" t="inlineStr">
@@ -4076,28 +4076,28 @@
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>Uyumsoft (.com)</t>
+          <t>Softtech</t>
         </is>
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>https://uyumsoft.com</t>
+          <t>https://www.softtech.com.tr</t>
         </is>
       </c>
       <c r="C97" s="2" t="inlineStr"/>
       <c r="D97" s="3" t="inlineStr">
         <is>
-          <t>ik@uyumsoft.com, kariyer@uyumsoft.com, career@uyumsoft.com, cv@uyumsoft.com</t>
+          <t>ik@softtech.com.tr, kariyer@softtech.com.tr, career@softtech.com.tr, cv@softtech.com.tr</t>
         </is>
       </c>
       <c r="E97" s="2" t="inlineStr">
         <is>
-          <t>ERP / e-dönüşüm yazılımı</t>
+          <t>Bankacılık yazılımı</t>
         </is>
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
-          <t>Kullanıcı listesi (05.08.2026 - 2. parti)</t>
+          <t>Ön liste (doğrulanmadı)</t>
         </is>
       </c>
       <c r="G97" s="3" t="inlineStr">
@@ -4107,35 +4107,35 @@
       </c>
       <c r="H97" s="2" t="inlineStr">
         <is>
-          <t>Microsoft 365</t>
+          <t>var</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>VeriPark</t>
+          <t>Solvoyo</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>https://www.veripark.com</t>
+          <t>https://solvoyo.com</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr"/>
       <c r="D98" s="3" t="inlineStr">
         <is>
-          <t>ik@veripark.com, kariyer@veripark.com, career@veripark.com, cv@veripark.com</t>
+          <t>ik@solvoyo.com, kariyer@solvoyo.com, career@solvoyo.com, cv@solvoyo.com</t>
         </is>
       </c>
       <c r="E98" s="2" t="inlineStr">
         <is>
-          <t>Bankacılık yazılımı</t>
+          <t>Tedarik zinciri planlama / yapay zeka</t>
         </is>
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Kullanıcı listesi (05.08.2026 - 2. parti)</t>
         </is>
       </c>
       <c r="G98" s="3" t="inlineStr">
@@ -4145,31 +4145,35 @@
       </c>
       <c r="H98" s="2" t="inlineStr">
         <is>
-          <t>Microsoft 365</t>
+          <t>Google Workspace</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>Verisoft</t>
+          <t>Spyke Games</t>
         </is>
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>https://verisoft.com</t>
+          <t>https://www.spykegames.com</t>
         </is>
       </c>
       <c r="C99" s="2" t="inlineStr"/>
       <c r="D99" s="3" t="inlineStr">
         <is>
-          <t>ik@verisoft.com, kariyer@verisoft.com, career@verisoft.com, cv@verisoft.com</t>
-        </is>
-      </c>
-      <c r="E99" s="2" t="inlineStr"/>
+          <t>ik@spykegames.com, kariyer@spykegames.com, career@spykegames.com, cv@spykegames.com</t>
+        </is>
+      </c>
+      <c r="E99" s="2" t="inlineStr">
+        <is>
+          <t>Mobil oyun</t>
+        </is>
+      </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>Kullanıcı listesi (05.08.2026 - 2. parti)</t>
+          <t>Ön liste (doğrulanmadı)</t>
         </is>
       </c>
       <c r="G99" s="3" t="inlineStr">
@@ -4186,28 +4190,28 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>Virgosol</t>
+          <t>T-Soft</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>https://virgosol.com</t>
+          <t>https://www.tsoft.com.tr</t>
         </is>
       </c>
       <c r="C100" s="2" t="inlineStr"/>
       <c r="D100" s="3" t="inlineStr">
         <is>
-          <t>ik@virgosol.com, kariyer@virgosol.com, career@virgosol.com, cv@virgosol.com</t>
+          <t>ik@tsoft.com.tr, kariyer@tsoft.com.tr, career@tsoft.com.tr, cv@tsoft.com.tr</t>
         </is>
       </c>
       <c r="E100" s="2" t="inlineStr">
         <is>
-          <t>Yazılım geliştirme</t>
+          <t>E-ticaret yazılımı</t>
         </is>
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>Kullanıcı listesi (05.08.2026)</t>
+          <t>Ön liste (doğrulanmadı)</t>
         </is>
       </c>
       <c r="G100" s="3" t="inlineStr">
@@ -4217,35 +4221,31 @@
       </c>
       <c r="H100" s="2" t="inlineStr">
         <is>
-          <t>Microsoft 365</t>
+          <t>var</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>Vispera</t>
+          <t>TankX</t>
         </is>
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>https://vispera.co</t>
+          <t>https://tankx.co</t>
         </is>
       </c>
       <c r="C101" s="2" t="inlineStr"/>
       <c r="D101" s="3" t="inlineStr">
         <is>
-          <t>ik@vispera.co, kariyer@vispera.co, career@vispera.co, cv@vispera.co</t>
-        </is>
-      </c>
-      <c r="E101" s="2" t="inlineStr">
-        <is>
-          <t>Yapay zeka / görüntü işleme</t>
-        </is>
-      </c>
+          <t>ik@tankx.co, kariyer@tankx.co, career@tankx.co, cv@tankx.co</t>
+        </is>
+      </c>
+      <c r="E101" s="2" t="inlineStr"/>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>Ön liste (doğrulanmadı)</t>
+          <t>Kullanıcı listesi (05.08.2026)</t>
         </is>
       </c>
       <c r="G101" s="3" t="inlineStr">
@@ -4255,35 +4255,35 @@
       </c>
       <c r="H101" s="2" t="inlineStr">
         <is>
-          <t>Microsoft 365</t>
+          <t>Google Workspace</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>VoltLines</t>
+          <t>Testinium</t>
         </is>
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>https://voltlines.com</t>
+          <t>https://testinium.com</t>
         </is>
       </c>
       <c r="C102" s="2" t="inlineStr"/>
       <c r="D102" s="3" t="inlineStr">
         <is>
-          <t>ik@voltlines.com, kariyer@voltlines.com, career@voltlines.com, cv@voltlines.com</t>
+          <t>ik@testinium.com, kariyer@testinium.com, career@testinium.com, cv@testinium.com</t>
         </is>
       </c>
       <c r="E102" s="2" t="inlineStr">
         <is>
-          <t>Kurumsal ulaşım teknolojisi</t>
+          <t>Test otomasyonu / yazılım kalite</t>
         </is>
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>Kullanıcı listesi (05.08.2026)</t>
+          <t>Ön liste (doğrulanmadı)</t>
         </is>
       </c>
       <c r="G102" s="3" t="inlineStr">
@@ -4293,30 +4293,30 @@
       </c>
       <c r="H102" s="2" t="inlineStr">
         <is>
-          <t>Google Workspace</t>
+          <t>Microsoft 365</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>Workcube</t>
+          <t>Ticimax</t>
         </is>
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>https://www.workcube.com</t>
+          <t>https://www.ticimax.com</t>
         </is>
       </c>
       <c r="C103" s="2" t="inlineStr"/>
       <c r="D103" s="3" t="inlineStr">
         <is>
-          <t>ik@workcube.com, kariyer@workcube.com, career@workcube.com, cv@workcube.com</t>
+          <t>ik@ticimax.com, kariyer@ticimax.com, career@ticimax.com, cv@ticimax.com</t>
         </is>
       </c>
       <c r="E103" s="2" t="inlineStr">
         <is>
-          <t>Kurumsal yazılım / ERP</t>
+          <t>E-ticaret altyapı yazılımı</t>
         </is>
       </c>
       <c r="F103" s="2" t="inlineStr">
@@ -4331,50 +4331,388 @@
       </c>
       <c r="H103" s="2" t="inlineStr">
         <is>
-          <t>Google Workspace</t>
+          <t>Microsoft 365</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>Yemeksepeti</t>
+          <t>Trendyol</t>
         </is>
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>https://www.yemeksepeti.com</t>
+          <t>https://www.trendyol.com</t>
         </is>
       </c>
       <c r="C104" s="2" t="inlineStr"/>
       <c r="D104" s="3" t="inlineStr">
         <is>
+          <t>ik@trendyol.com, kariyer@trendyol.com, career@trendyol.com, cv@trendyol.com</t>
+        </is>
+      </c>
+      <c r="E104" s="2" t="inlineStr">
+        <is>
+          <t>E-ticaret platformu</t>
+        </is>
+      </c>
+      <c r="F104" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G104" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
+        </is>
+      </c>
+      <c r="H104" s="2" t="inlineStr">
+        <is>
+          <t>var</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="2" t="inlineStr">
+        <is>
+          <t>Uyumsoft</t>
+        </is>
+      </c>
+      <c r="B105" s="2" t="inlineStr">
+        <is>
+          <t>https://www.uyumsoft.com.tr</t>
+        </is>
+      </c>
+      <c r="C105" s="2" t="inlineStr"/>
+      <c r="D105" s="3" t="inlineStr">
+        <is>
+          <t>ik@uyumsoft.com.tr, kariyer@uyumsoft.com.tr, career@uyumsoft.com.tr, cv@uyumsoft.com.tr</t>
+        </is>
+      </c>
+      <c r="E105" s="2" t="inlineStr">
+        <is>
+          <t>ERP / e-dönüşüm yazılımı</t>
+        </is>
+      </c>
+      <c r="F105" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G105" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
+        </is>
+      </c>
+      <c r="H105" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft 365</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="2" t="inlineStr">
+        <is>
+          <t>Uyumsoft (.com)</t>
+        </is>
+      </c>
+      <c r="B106" s="2" t="inlineStr">
+        <is>
+          <t>https://uyumsoft.com</t>
+        </is>
+      </c>
+      <c r="C106" s="2" t="inlineStr"/>
+      <c r="D106" s="3" t="inlineStr">
+        <is>
+          <t>ik@uyumsoft.com, kariyer@uyumsoft.com, career@uyumsoft.com, cv@uyumsoft.com</t>
+        </is>
+      </c>
+      <c r="E106" s="2" t="inlineStr">
+        <is>
+          <t>ERP / e-dönüşüm yazılımı</t>
+        </is>
+      </c>
+      <c r="F106" s="2" t="inlineStr">
+        <is>
+          <t>Kullanıcı listesi (05.08.2026 - 2. parti)</t>
+        </is>
+      </c>
+      <c r="G106" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
+        </is>
+      </c>
+      <c r="H106" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft 365</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="2" t="inlineStr">
+        <is>
+          <t>VeriPark</t>
+        </is>
+      </c>
+      <c r="B107" s="2" t="inlineStr">
+        <is>
+          <t>https://www.veripark.com</t>
+        </is>
+      </c>
+      <c r="C107" s="2" t="inlineStr"/>
+      <c r="D107" s="3" t="inlineStr">
+        <is>
+          <t>ik@veripark.com, kariyer@veripark.com, career@veripark.com, cv@veripark.com</t>
+        </is>
+      </c>
+      <c r="E107" s="2" t="inlineStr">
+        <is>
+          <t>Bankacılık yazılımı</t>
+        </is>
+      </c>
+      <c r="F107" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G107" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
+        </is>
+      </c>
+      <c r="H107" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft 365</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="inlineStr">
+        <is>
+          <t>Verisoft</t>
+        </is>
+      </c>
+      <c r="B108" s="2" t="inlineStr">
+        <is>
+          <t>https://verisoft.com</t>
+        </is>
+      </c>
+      <c r="C108" s="2" t="inlineStr"/>
+      <c r="D108" s="3" t="inlineStr">
+        <is>
+          <t>ik@verisoft.com, kariyer@verisoft.com, career@verisoft.com, cv@verisoft.com</t>
+        </is>
+      </c>
+      <c r="E108" s="2" t="inlineStr"/>
+      <c r="F108" s="2" t="inlineStr">
+        <is>
+          <t>Kullanıcı listesi (05.08.2026 - 2. parti)</t>
+        </is>
+      </c>
+      <c r="G108" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
+        </is>
+      </c>
+      <c r="H108" s="2" t="inlineStr">
+        <is>
+          <t>Google Workspace</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="2" t="inlineStr">
+        <is>
+          <t>Virgosol</t>
+        </is>
+      </c>
+      <c r="B109" s="2" t="inlineStr">
+        <is>
+          <t>https://virgosol.com</t>
+        </is>
+      </c>
+      <c r="C109" s="2" t="inlineStr"/>
+      <c r="D109" s="3" t="inlineStr">
+        <is>
+          <t>ik@virgosol.com, kariyer@virgosol.com, career@virgosol.com, cv@virgosol.com</t>
+        </is>
+      </c>
+      <c r="E109" s="2" t="inlineStr">
+        <is>
+          <t>Yazılım geliştirme</t>
+        </is>
+      </c>
+      <c r="F109" s="2" t="inlineStr">
+        <is>
+          <t>Kullanıcı listesi (05.08.2026)</t>
+        </is>
+      </c>
+      <c r="G109" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
+        </is>
+      </c>
+      <c r="H109" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft 365</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="inlineStr">
+        <is>
+          <t>Vispera</t>
+        </is>
+      </c>
+      <c r="B110" s="2" t="inlineStr">
+        <is>
+          <t>https://vispera.co</t>
+        </is>
+      </c>
+      <c r="C110" s="2" t="inlineStr"/>
+      <c r="D110" s="3" t="inlineStr">
+        <is>
+          <t>ik@vispera.co, kariyer@vispera.co, career@vispera.co, cv@vispera.co</t>
+        </is>
+      </c>
+      <c r="E110" s="2" t="inlineStr">
+        <is>
+          <t>Yapay zeka / görüntü işleme</t>
+        </is>
+      </c>
+      <c r="F110" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G110" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
+        </is>
+      </c>
+      <c r="H110" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft 365</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="2" t="inlineStr">
+        <is>
+          <t>VoltLines</t>
+        </is>
+      </c>
+      <c r="B111" s="2" t="inlineStr">
+        <is>
+          <t>https://voltlines.com</t>
+        </is>
+      </c>
+      <c r="C111" s="2" t="inlineStr"/>
+      <c r="D111" s="3" t="inlineStr">
+        <is>
+          <t>ik@voltlines.com, kariyer@voltlines.com, career@voltlines.com, cv@voltlines.com</t>
+        </is>
+      </c>
+      <c r="E111" s="2" t="inlineStr">
+        <is>
+          <t>Kurumsal ulaşım teknolojisi</t>
+        </is>
+      </c>
+      <c r="F111" s="2" t="inlineStr">
+        <is>
+          <t>Kullanıcı listesi (05.08.2026)</t>
+        </is>
+      </c>
+      <c r="G111" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
+        </is>
+      </c>
+      <c r="H111" s="2" t="inlineStr">
+        <is>
+          <t>Google Workspace</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="2" t="inlineStr">
+        <is>
+          <t>Workcube</t>
+        </is>
+      </c>
+      <c r="B112" s="2" t="inlineStr">
+        <is>
+          <t>https://www.workcube.com</t>
+        </is>
+      </c>
+      <c r="C112" s="2" t="inlineStr"/>
+      <c r="D112" s="3" t="inlineStr">
+        <is>
+          <t>ik@workcube.com, kariyer@workcube.com, career@workcube.com, cv@workcube.com</t>
+        </is>
+      </c>
+      <c r="E112" s="2" t="inlineStr">
+        <is>
+          <t>Kurumsal yazılım / ERP</t>
+        </is>
+      </c>
+      <c r="F112" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G112" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
+        </is>
+      </c>
+      <c r="H112" s="2" t="inlineStr">
+        <is>
+          <t>Google Workspace</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="2" t="inlineStr">
+        <is>
+          <t>Yemeksepeti</t>
+        </is>
+      </c>
+      <c r="B113" s="2" t="inlineStr">
+        <is>
+          <t>https://www.yemeksepeti.com</t>
+        </is>
+      </c>
+      <c r="C113" s="2" t="inlineStr"/>
+      <c r="D113" s="3" t="inlineStr">
+        <is>
           <t>ik@yemeksepeti.com, kariyer@yemeksepeti.com, career@yemeksepeti.com, cv@yemeksepeti.com</t>
         </is>
       </c>
-      <c r="E104" s="2" t="inlineStr">
+      <c r="E113" s="2" t="inlineStr">
         <is>
           <t>Online yemek siparişi</t>
         </is>
       </c>
-      <c r="F104" s="2" t="inlineStr">
-        <is>
-          <t>Ön liste (doğrulanmadı)</t>
-        </is>
-      </c>
-      <c r="G104" s="3" t="inlineStr">
-        <is>
-          <t>üretildi – doğrulanmadı</t>
-        </is>
-      </c>
-      <c r="H104" s="2" t="inlineStr">
+      <c r="F113" s="2" t="inlineStr">
+        <is>
+          <t>Ön liste (doğrulanmadı)</t>
+        </is>
+      </c>
+      <c r="G113" s="3" t="inlineStr">
+        <is>
+          <t>üretildi – doğrulanmadı</t>
+        </is>
+      </c>
+      <c r="H113" s="2" t="inlineStr">
         <is>
           <t>Google Workspace</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H104"/>
+  <autoFilter ref="A1:H113"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>